<commit_message>
fix: harden installer upload and dedupe seo keywords
</commit_message>
<xml_diff>
--- a/shared/data/categories_import.xlsx
+++ b/shared/data/categories_import.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="171">
   <si>
     <t>category_id</t>
   </si>
@@ -526,6 +526,9 @@
   </si>
   <si>
     <t>dobriva-ta-stimuliatori</t>
+  </si>
+  <si>
+    <t>fungitsidi-408</t>
   </si>
 </sst>
 </file>
@@ -2808,7 +2811,7 @@
         <v>0</v>
       </c>
       <c r="C42" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: drop category 408 from dataset
</commit_message>
<xml_diff>
--- a/shared/data/categories_import.xlsx
+++ b/shared/data/categories_import.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="169">
   <si>
     <t>category_id</t>
   </si>
@@ -393,9 +393,6 @@
     <t>c407.jpg</t>
   </si>
   <si>
-    <t>c408.jpg</t>
-  </si>
-  <si>
     <t>Супутні товари</t>
   </si>
   <si>
@@ -526,9 +523,6 @@
   </si>
   <si>
     <t>dobriva-ta-stimuliatori</t>
-  </si>
-  <si>
-    <t>fungitsidi-408</t>
   </si>
 </sst>
 </file>
@@ -864,7 +858,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:12">
@@ -2265,65 +2259,31 @@
     </row>
     <row r="42" spans="1:12">
       <c r="A42">
-        <v>408</v>
+        <v>500</v>
       </c>
       <c r="B42">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="C42" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D42">
         <v>41</v>
       </c>
       <c r="E42" t="s">
+        <v>126</v>
+      </c>
+      <c r="F42"/>
+      <c r="G42" t="s">
         <v>125</v>
       </c>
-      <c r="F42" t="s">
-        <v>123</v>
-      </c>
-      <c r="G42" t="s">
-        <v>117</v>
-      </c>
-      <c r="H42" t="s">
-        <v>123</v>
-      </c>
+      <c r="H42"/>
       <c r="I42"/>
       <c r="J42">
         <v>0</v>
       </c>
       <c r="K42"/>
       <c r="L42" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12">
-      <c r="A43">
-        <v>500</v>
-      </c>
-      <c r="B43">
-        <v>0</v>
-      </c>
-      <c r="C43" t="s">
-        <v>126</v>
-      </c>
-      <c r="D43">
-        <v>42</v>
-      </c>
-      <c r="E43" t="s">
-        <v>127</v>
-      </c>
-      <c r="F43"/>
-      <c r="G43" t="s">
-        <v>126</v>
-      </c>
-      <c r="H43"/>
-      <c r="I43"/>
-      <c r="J43">
-        <v>0</v>
-      </c>
-      <c r="K43"/>
-      <c r="L43" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2349,7 +2309,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2357,10 +2317,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C1" t="s">
         <v>128</v>
-      </c>
-      <c r="C1" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -2371,7 +2331,7 @@
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2382,7 +2342,7 @@
         <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2393,7 +2353,7 @@
         <v>0</v>
       </c>
       <c r="C4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -2404,7 +2364,7 @@
         <v>0</v>
       </c>
       <c r="C5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -2415,7 +2375,7 @@
         <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -2426,7 +2386,7 @@
         <v>0</v>
       </c>
       <c r="C7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -2437,7 +2397,7 @@
         <v>0</v>
       </c>
       <c r="C8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -2448,7 +2408,7 @@
         <v>0</v>
       </c>
       <c r="C9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -2459,7 +2419,7 @@
         <v>0</v>
       </c>
       <c r="C10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -2470,7 +2430,7 @@
         <v>0</v>
       </c>
       <c r="C11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -2481,7 +2441,7 @@
         <v>0</v>
       </c>
       <c r="C12" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -2492,7 +2452,7 @@
         <v>0</v>
       </c>
       <c r="C13" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -2503,7 +2463,7 @@
         <v>0</v>
       </c>
       <c r="C14" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -2514,7 +2474,7 @@
         <v>0</v>
       </c>
       <c r="C15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -2525,7 +2485,7 @@
         <v>0</v>
       </c>
       <c r="C16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -2536,7 +2496,7 @@
         <v>0</v>
       </c>
       <c r="C17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -2547,7 +2507,7 @@
         <v>0</v>
       </c>
       <c r="C18" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -2558,7 +2518,7 @@
         <v>0</v>
       </c>
       <c r="C19" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -2569,7 +2529,7 @@
         <v>0</v>
       </c>
       <c r="C20" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -2580,7 +2540,7 @@
         <v>0</v>
       </c>
       <c r="C21" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -2591,7 +2551,7 @@
         <v>0</v>
       </c>
       <c r="C22" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -2602,7 +2562,7 @@
         <v>0</v>
       </c>
       <c r="C23" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -2613,7 +2573,7 @@
         <v>0</v>
       </c>
       <c r="C24" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -2624,7 +2584,7 @@
         <v>0</v>
       </c>
       <c r="C25" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -2635,7 +2595,7 @@
         <v>0</v>
       </c>
       <c r="C26" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -2646,7 +2606,7 @@
         <v>0</v>
       </c>
       <c r="C27" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -2657,7 +2617,7 @@
         <v>0</v>
       </c>
       <c r="C28" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -2668,7 +2628,7 @@
         <v>0</v>
       </c>
       <c r="C29" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -2679,7 +2639,7 @@
         <v>0</v>
       </c>
       <c r="C30" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -2690,7 +2650,7 @@
         <v>0</v>
       </c>
       <c r="C31" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -2701,7 +2661,7 @@
         <v>0</v>
       </c>
       <c r="C32" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -2712,7 +2672,7 @@
         <v>0</v>
       </c>
       <c r="C33" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -2723,7 +2683,7 @@
         <v>0</v>
       </c>
       <c r="C34" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -2734,7 +2694,7 @@
         <v>0</v>
       </c>
       <c r="C35" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -2745,7 +2705,7 @@
         <v>0</v>
       </c>
       <c r="C36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -2756,7 +2716,7 @@
         <v>0</v>
       </c>
       <c r="C37" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -2767,7 +2727,7 @@
         <v>0</v>
       </c>
       <c r="C38" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -2778,7 +2738,7 @@
         <v>0</v>
       </c>
       <c r="C39" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -2789,7 +2749,7 @@
         <v>0</v>
       </c>
       <c r="C40" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -2800,18 +2760,7 @@
         <v>0</v>
       </c>
       <c r="C41" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3">
-      <c r="A42">
-        <v>408</v>
-      </c>
-      <c r="B42">
-        <v>0</v>
-      </c>
-      <c r="C42" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: point category images to catalog/categories
</commit_message>
<xml_diff>
--- a/shared/data/categories_import.xlsx
+++ b/shared/data/categories_import.xlsx
@@ -57,7 +57,7 @@
     <t>Томати</t>
   </si>
   <si>
-    <t>c100.jpg</t>
+    <t>catalog/categories/c100.jpg</t>
   </si>
   <si>
     <t>Томати відносяться до роду пасльонових. Рослина рясніє великою кількістю сортів. Поширений овоч по всьому світу.</t>
@@ -69,7 +69,7 @@
     <t>Томати високорослі</t>
   </si>
   <si>
-    <t>c101.jpg</t>
+    <t>catalog/categories/c101.jpg</t>
   </si>
   <si>
     <t>Відмітна риса високорослих томатів, висота стебла іноді досягає 2,50 м, цим обумовлюється велика віддача врожаю. Іноді з куща можна зняти до 8 кг плодів.</t>
@@ -78,7 +78,7 @@
     <t>Томати середньорослі</t>
   </si>
   <si>
-    <t>c102.jpg</t>
+    <t>catalog/categories/c102.jpg</t>
   </si>
   <si>
     <t>Середньорослі томати зібрали в собі найкращі якості високорослих і низькорослих сортів, зазвичай вирощуються в два стебла.</t>
@@ -87,7 +87,7 @@
     <t>Томати низькорослі</t>
   </si>
   <si>
-    <t>c103.jpg</t>
+    <t>catalog/categories/c103.jpg</t>
   </si>
   <si>
     <t>Низькорослі сорти томатів відрізняються швидкою віддачею, формуючи невелику кількість кистей, дружним дозріванням.</t>
@@ -96,7 +96,7 @@
     <t>Огірки</t>
   </si>
   <si>
-    <t>c110.jpg</t>
+    <t>catalog/categories/c110.jpg</t>
   </si>
   <si>
     <t>Найпопулярнійшої овочевий продукт, який можна випращівать цілий рік. Невибагливий, а так же незамінний в салатах.</t>
@@ -105,7 +105,7 @@
     <t>Капуста</t>
   </si>
   <si>
-    <t>c120.jpg</t>
+    <t>catalog/categories/c120.jpg</t>
   </si>
   <si>
     <t>Капуста - цариця серед овочів, дуже популярний продукт. Займає одне з перших місць в світі по вирощуванню.</t>
@@ -114,7 +114,7 @@
     <t>Капуста білокачанна</t>
   </si>
   <si>
-    <t>c121.jpg</t>
+    <t>catalog/categories/c121.jpg</t>
   </si>
   <si>
     <t>Різновид сімейства хрестоцвітних. Налічує близько 400 сортів різних термінів дозрівання.</t>
@@ -123,7 +123,7 @@
     <t>Капуста цвітна</t>
   </si>
   <si>
-    <t>c122.jpg</t>
+    <t>catalog/categories/c122.jpg</t>
   </si>
   <si>
     <t>Цвітна капуста має однорічний цикл розвитку, різноманіття сортів дивує своєю незвичністю. Має високі смакові якості.</t>
@@ -132,7 +132,7 @@
     <t>Капуста червонокачанна</t>
   </si>
   <si>
-    <t>c123.jpg</t>
+    <t>catalog/categories/c123.jpg</t>
   </si>
   <si>
     <t>Це вид капусти містить велику кількість макро і мікро елементів, стійкий до захворювань, добре зберігається і дуже смачний в салатах.</t>
@@ -147,7 +147,7 @@
     <t>Редис</t>
   </si>
   <si>
-    <t>c130.jpg</t>
+    <t>catalog/categories/c130.jpg</t>
   </si>
   <si>
     <t>Редис характерний ранніми термінами дозрівання, саме з нього роблять перші салати після зими.</t>
@@ -156,7 +156,7 @@
     <t>Перець</t>
   </si>
   <si>
-    <t>c140.jpg</t>
+    <t>catalog/categories/c140.jpg</t>
   </si>
   <si>
     <t>Будь-яка кухня світу використовує перець, як необхідний компонент перших і других страв. Високий вміст вітаміну С, а так само інших корисних мікроелементів робить його незамінним.</t>
@@ -165,7 +165,7 @@
     <t>Перець солодкий</t>
   </si>
   <si>
-    <t>c141.jpg</t>
+    <t>catalog/categories/c141.jpg</t>
   </si>
   <si>
     <t>Солодкі перці мають дуже привабливий вигляд. М'ясисті і смачні.</t>
@@ -174,7 +174,7 @@
     <t>Перець гіркий</t>
   </si>
   <si>
-    <t>c142.jpg</t>
+    <t>catalog/categories/c142.jpg</t>
   </si>
   <si>
     <t>Культурних сортів гострого перцю близько 3000. Добре зберігається в сушеному вигляді.</t>
@@ -183,7 +183,7 @@
     <t>Баклажани</t>
   </si>
   <si>
-    <t>c150.jpg</t>
+    <t>catalog/categories/c150.jpg</t>
   </si>
   <si>
     <t>Ця рослина ставитися до роду пасльонових і вирощується як однорічник. У їжу вживають злегка недозрілі плоди так вони смачніші.</t>
@@ -192,7 +192,7 @@
     <t>Цибуля</t>
   </si>
   <si>
-    <t>c160.jpg</t>
+    <t>catalog/categories/c160.jpg</t>
   </si>
   <si>
     <t>Різноманітність сортів луків не припиняє дивувати: однорічні, дворічні і навіть багаторічні. Багаті зеленню обеспечиват вітамінами круглий рік.</t>
@@ -201,7 +201,7 @@
     <t>Морква</t>
   </si>
   <si>
-    <t>c170.jpg</t>
+    <t>catalog/categories/c170.jpg</t>
   </si>
   <si>
     <t>Морква містить масу корисних речовин - це каротин, солі, калію, пектини, вітаміни А, В, С, Д. Широко застосовується в кулінарії, не замінна в дитячому харчуванні.</t>
@@ -210,7 +210,7 @@
     <t>Буряк</t>
   </si>
   <si>
-    <t>c180.jpg</t>
+    <t>catalog/categories/c180.jpg</t>
   </si>
   <si>
     <t>Буряк має дуже високими смаковими і лікувальними властивостями, збагачена йодом, вітамінами А і В, покращує обмін речовин. У деяких сортів використовують і коренеплоди і надземну частину.</t>
@@ -219,7 +219,7 @@
     <t>Кавуни</t>
   </si>
   <si>
-    <t>c190.jpg</t>
+    <t>catalog/categories/c190.jpg</t>
   </si>
   <si>
     <t>Рослина поширилося з Африки, пройшло довгий селекційний шлях. На сьогодні це - однорічна стелеться трава з кавалками листям. Плід кавуна - соковита ягода з безліччю насіння.</t>
@@ -228,7 +228,7 @@
     <t>Дині</t>
   </si>
   <si>
-    <t>c200.jpg</t>
+    <t>catalog/categories/c200.jpg</t>
   </si>
   <si>
     <t>Традиційна баштанних культур для степової зони. Головне дати рослині більше тепла і сонця. Урожай, при дотриманні агротехніки обробітку, можна отримати вже в кінці червня.</t>
@@ -237,7 +237,7 @@
     <t>Гарбузи</t>
   </si>
   <si>
-    <t>c210.jpg</t>
+    <t>catalog/categories/c210.jpg</t>
   </si>
   <si>
     <t>За кількістю вмісту заліза, гарбуз - чемпіон серед овочів. Гарбузове насіння джерело масел, багатих мікроелементами. Її соковита м'якоть використовується в дієтології.</t>
@@ -246,7 +246,7 @@
     <t>Кабачки</t>
   </si>
   <si>
-    <t>c220.jpg</t>
+    <t>catalog/categories/c220.jpg</t>
   </si>
   <si>
     <t>Кабачок - цукіні продукт, низькокалорійний і легкозасвоюваний організмом, тому його використовують в дієтології і в дитячому харчуванні.</t>
@@ -255,7 +255,7 @@
     <t>Патисони</t>
   </si>
   <si>
-    <t>c230.jpg</t>
+    <t>catalog/categories/c230.jpg</t>
   </si>
   <si>
     <t>Плоди патисонів тонкокорие. М'якоть білосніжна, хрустка і дуже щільна. Малюками зазвичай підходять для консервації, а більші плоди використовують в кулінарії.</t>
@@ -264,7 +264,7 @@
     <t>Зелені культури</t>
   </si>
   <si>
-    <t>c240.jpg</t>
+    <t>catalog/categories/c240.jpg</t>
   </si>
   <si>
     <t>Ранні вітаміни на столах - зелені культури. Всі різновиди салатів, шпинат, щавель, спаржа, черемша.</t>
@@ -273,7 +273,7 @@
     <t>Пряносмакові культури</t>
   </si>
   <si>
-    <t>c250.jpg</t>
+    <t>catalog/categories/c250.jpg</t>
   </si>
   <si>
     <t>До групи пряно-смакових культур входять трави, які використовуються як приправи: майоран, кріп, чабер і багато-багато інших однорічних і багаторічних рослин. Вони відносно холодостійкі.</t>
@@ -282,7 +282,7 @@
     <t>Бобові культури</t>
   </si>
   <si>
-    <t>c270.jpg</t>
+    <t>catalog/categories/c270.jpg</t>
   </si>
   <si>
     <t>Різноманітність видів сімейства бобових - величезна. Застосовують їх як продукт харчування.</t>
@@ -291,7 +291,7 @@
     <t>Квасоля</t>
   </si>
   <si>
-    <t>c280.jpg</t>
+    <t>catalog/categories/c280.jpg</t>
   </si>
   <si>
     <t>Квасоля відноситься до розряду бобових з за того, що має стручкову форму заповнену зернами і тим не менше це відмінне від бобових рослина, що має дуже багато різних сортів.</t>
@@ -300,7 +300,7 @@
     <t>Квасоля спаржева</t>
   </si>
   <si>
-    <t>c281.jpg</t>
+    <t>catalog/categories/c281.jpg</t>
   </si>
   <si>
     <t>Спаржева квасоля вирощується заради смачних стулок: у них відсутній пергаментний прошарок, тому квасоля вживається в їжу цілком. Смаком нагадує спаржу.</t>
@@ -309,7 +309,7 @@
     <t>Квасоля зернова</t>
   </si>
   <si>
-    <t>c282.jpg</t>
+    <t>catalog/categories/c282.jpg</t>
   </si>
   <si>
     <t>Лущильні сорти квасолі вирощуються виключно для вживання в їжу зерен: дуже поживних і містять велику кількість білка.</t>
@@ -318,7 +318,7 @@
     <t>Кукурудза</t>
   </si>
   <si>
-    <t>c290.jpg</t>
+    <t>catalog/categories/c290.jpg</t>
   </si>
   <si>
     <t>Кукурудза - цариця полів, це однорічна трав'яниста рослина відноситься до злакових культур.</t>
@@ -327,7 +327,7 @@
     <t>Квіти</t>
   </si>
   <si>
-    <t>c330.jpg</t>
+    <t>catalog/categories/c330.jpg</t>
   </si>
   <si>
     <t>Аромати, різноманітність кольору, ніжність, трепет і любов - все це відноситься до багатотисячної армії квітів всіх видів, всіх категорій і всіх національностей.</t>
@@ -336,7 +336,7 @@
     <t>Квіти однорічні</t>
   </si>
   <si>
-    <t>c331.jpg</t>
+    <t>catalog/categories/c331.jpg</t>
   </si>
   <si>
     <t>Великий діапазон кольорів, багатий вибір форм, різниця термінів цвітіння - дає можливість створювати будь-які композиції. І те, що рослини однорічні - дозволяє експериментувати нескінченно.</t>
@@ -345,7 +345,7 @@
     <t>Квіти багаторічні</t>
   </si>
   <si>
-    <t>c332.jpg</t>
+    <t>catalog/categories/c332.jpg</t>
   </si>
   <si>
     <t>Багаторічники зазвичай дають можливість формувати композиції на кілька років вперед. Прекрасно сусідять зі своїми побратимами і не вибагливі до ґрунту. Це і високорослі, і цибулинні (типу мускари або птицемлечник), і стелящиеся почвопокривні рослини.</t>
@@ -354,49 +354,49 @@
     <t>Добрива та захист</t>
   </si>
   <si>
-    <t>c400.jpg</t>
+    <t>catalog/categories/c400.jpg</t>
   </si>
   <si>
     <t>Гербіциди</t>
   </si>
   <si>
-    <t>c401.jpg</t>
+    <t>catalog/categories/c401.jpg</t>
   </si>
   <si>
     <t>Інсектициди</t>
   </si>
   <si>
-    <t>c402.jpg</t>
+    <t>catalog/categories/c402.jpg</t>
   </si>
   <si>
     <t>Фунгіциди</t>
   </si>
   <si>
-    <t>c403.jpg</t>
+    <t>catalog/categories/c403.jpg</t>
   </si>
   <si>
     <t>Біопрепарати</t>
   </si>
   <si>
-    <t>c405.jpg</t>
+    <t>catalog/categories/c405.jpg</t>
   </si>
   <si>
     <t>Прилипачі</t>
   </si>
   <si>
-    <t>c406.jpg</t>
+    <t>catalog/categories/c406.jpg</t>
   </si>
   <si>
     <t>Добрива та стимулятори</t>
   </si>
   <si>
-    <t>c407.jpg</t>
+    <t>catalog/categories/c407.jpg</t>
   </si>
   <si>
     <t>Супутні товари</t>
   </si>
   <si>
-    <t>c500.jpg</t>
+    <t>catalog/categories/c500.jpg</t>
   </si>
   <si>
     <t>store_id</t>

</xml_diff>

<commit_message>
feat: add uk-ua content and better transliteration
</commit_message>
<xml_diff>
--- a/shared/data/categories_import.xlsx
+++ b/shared/data/categories_import.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="249">
   <si>
     <t>category_id</t>
   </si>
@@ -27,6 +27,9 @@
     <t>name(en-gb)</t>
   </si>
   <si>
+    <t>name(uk-ua)</t>
+  </si>
+  <si>
     <t>sort_order</t>
   </si>
   <si>
@@ -36,15 +39,27 @@
     <t>description(en-gb)</t>
   </si>
   <si>
+    <t>description(uk-ua)</t>
+  </si>
+  <si>
     <t>meta_title(en-gb)</t>
   </si>
   <si>
+    <t>meta_title(uk-ua)</t>
+  </si>
+  <si>
     <t>meta_description(en-gb)</t>
   </si>
   <si>
+    <t>meta_description(uk-ua)</t>
+  </si>
+  <si>
     <t>meta_keywords(en-gb)</t>
   </si>
   <si>
+    <t>meta_keywords(uk-ua)</t>
+  </si>
+  <si>
     <t>store_ids</t>
   </si>
   <si>
@@ -54,345 +69,567 @@
     <t>status</t>
   </si>
   <si>
+    <t>Tomaty</t>
+  </si>
+  <si>
     <t>Томати</t>
   </si>
   <si>
     <t>catalog/categories/c100.jpg</t>
   </si>
   <si>
+    <t>Tomaty vidnosyatsya do rodu paslonovykh. Roslyna ryasniie velykoyu kilkistyu sortiv. Poshyrenyi ovoch po vsomu svitu.</t>
+  </si>
+  <si>
     <t>Томати відносяться до роду пасльонових. Рослина рясніє великою кількістю сортів. Поширений овоч по всьому світу.</t>
   </si>
   <si>
     <t>true</t>
   </si>
   <si>
+    <t>Tomaty vysokorosli</t>
+  </si>
+  <si>
     <t>Томати високорослі</t>
   </si>
   <si>
     <t>catalog/categories/c101.jpg</t>
   </si>
   <si>
+    <t>Vidmitna rysa vysokoroslykh tomativ, vysota stebla inodi dosyahaie 2,50 m, tsym obumovlyuietsya velyka viddacha vrozhayu. Inodi z kushcha mozhna znyaty do 8 kh plodiv.</t>
+  </si>
+  <si>
     <t>Відмітна риса високорослих томатів, висота стебла іноді досягає 2,50 м, цим обумовлюється велика віддача врожаю. Іноді з куща можна зняти до 8 кг плодів.</t>
   </si>
   <si>
+    <t>Tomaty serednorosli</t>
+  </si>
+  <si>
     <t>Томати середньорослі</t>
   </si>
   <si>
     <t>catalog/categories/c102.jpg</t>
   </si>
   <si>
+    <t>Serednorosli tomaty zibraly v sobi naikrashchi yakosti vysokoroslykh i nyzkoroslykh sortiv, zazvychai vyroshchuyutsya v dva stebla.</t>
+  </si>
+  <si>
     <t>Середньорослі томати зібрали в собі найкращі якості високорослих і низькорослих сортів, зазвичай вирощуються в два стебла.</t>
   </si>
   <si>
+    <t>Tomaty nyzkorosli</t>
+  </si>
+  <si>
     <t>Томати низькорослі</t>
   </si>
   <si>
     <t>catalog/categories/c103.jpg</t>
   </si>
   <si>
+    <t>Nyzkorosli sorty tomativ vidriznyayutsya shvydkoyu viddacheyu, formuyuchy nevelyku kilkist kystei, druzhnym dozrivannyam.</t>
+  </si>
+  <si>
     <t>Низькорослі сорти томатів відрізняються швидкою віддачею, формуючи невелику кількість кистей, дружним дозріванням.</t>
   </si>
   <si>
+    <t>Ohirky</t>
+  </si>
+  <si>
     <t>Огірки</t>
   </si>
   <si>
     <t>catalog/categories/c110.jpg</t>
   </si>
   <si>
+    <t>Naipopulyarniishoi ovochevyi produkt, yakyi mozhna vyprashchivat tsilyi rik. Nevybahlyvyi, a tak zhe nezaminnyi v salatakh.</t>
+  </si>
+  <si>
     <t>Найпопулярнійшої овочевий продукт, який можна випращівать цілий рік. Невибагливий, а так же незамінний в салатах.</t>
   </si>
   <si>
+    <t>Kapusta</t>
+  </si>
+  <si>
     <t>Капуста</t>
   </si>
   <si>
     <t>catalog/categories/c120.jpg</t>
   </si>
   <si>
+    <t>Kapusta - tsarytsya sered ovochiv, duzhe populyarnyi produkt. Zaimaie odne z pershykh mists v sviti po vyroshchuvannyu.</t>
+  </si>
+  <si>
     <t>Капуста - цариця серед овочів, дуже популярний продукт. Займає одне з перших місць в світі по вирощуванню.</t>
   </si>
   <si>
+    <t>Kapusta bilokachanna</t>
+  </si>
+  <si>
     <t>Капуста білокачанна</t>
   </si>
   <si>
     <t>catalog/categories/c121.jpg</t>
   </si>
   <si>
+    <t>Riznovyd simeistva khrestotsvitnykh. Nalichuie blyzko 400 sortiv riznykh terminiv dozrivannya.</t>
+  </si>
+  <si>
     <t>Різновид сімейства хрестоцвітних. Налічує близько 400 сортів різних термінів дозрівання.</t>
   </si>
   <si>
+    <t>Kapusta tsvitna</t>
+  </si>
+  <si>
     <t>Капуста цвітна</t>
   </si>
   <si>
     <t>catalog/categories/c122.jpg</t>
   </si>
   <si>
+    <t>Tsvitna kapusta maie odnorichnyi tsykl rozvytku, riznomanittya sortiv dyvuie svoieyu nezvychnistyu. Maie vysoki smakovi yakosti.</t>
+  </si>
+  <si>
     <t>Цвітна капуста має однорічний цикл розвитку, різноманіття сортів дивує своєю незвичністю. Має високі смакові якості.</t>
   </si>
   <si>
+    <t>Kapusta chervonokachanna</t>
+  </si>
+  <si>
     <t>Капуста червонокачанна</t>
   </si>
   <si>
     <t>catalog/categories/c123.jpg</t>
   </si>
   <si>
+    <t>Tse vyd kapusty mistyt velyku kilkist makro i mikro elementiv, stiikyi do zakhvoryuvan, dobre zberihaietsya i duzhe smachnyi v salatakh.</t>
+  </si>
+  <si>
     <t>Це вид капусти містить велику кількість макро і мікро елементів, стійкий до захворювань, добре зберігається і дуже смачний в салатах.</t>
   </si>
   <si>
+    <t>Riznovydy kapusty</t>
+  </si>
+  <si>
     <t>Різновиди капусти</t>
   </si>
   <si>
+    <t>Riznovydiv isnuie bahato i vsi vony razyuche vidriznyayutsya odyn vid odnoho, ale obiednuie ikh odne - vsi vony kapusta.</t>
+  </si>
+  <si>
     <t>Різновидів існує багато і всі вони разюче відрізняються один від одного, але об'єднує їх одне - всі вони капуста.</t>
   </si>
   <si>
+    <t>Redys</t>
+  </si>
+  <si>
     <t>Редис</t>
   </si>
   <si>
     <t>catalog/categories/c130.jpg</t>
   </si>
   <si>
+    <t>Redys kharakternyi rannimy terminamy dozrivannya, same z noho roblyat pershi salaty pislya zymy.</t>
+  </si>
+  <si>
     <t>Редис характерний ранніми термінами дозрівання, саме з нього роблять перші салати після зими.</t>
   </si>
   <si>
+    <t>Perets</t>
+  </si>
+  <si>
     <t>Перець</t>
   </si>
   <si>
     <t>catalog/categories/c140.jpg</t>
   </si>
   <si>
+    <t>Bud-yaka kukhnya svitu vykorystovuie perets, yak neobkhidnyi komponent pershykh i druhykh strav. Vysokyi vmist vitaminu S, a tak samo inshykh korysnykh mikroelementiv robyt ioho nezaminnym.</t>
+  </si>
+  <si>
     <t>Будь-яка кухня світу використовує перець, як необхідний компонент перших і других страв. Високий вміст вітаміну С, а так само інших корисних мікроелементів робить його незамінним.</t>
   </si>
   <si>
+    <t>Perets solodkyi</t>
+  </si>
+  <si>
     <t>Перець солодкий</t>
   </si>
   <si>
     <t>catalog/categories/c141.jpg</t>
   </si>
   <si>
+    <t>Solodki pertsi mayut duzhe pryvablyvyi vyhlyad. Myasysti i smachni.</t>
+  </si>
+  <si>
     <t>Солодкі перці мають дуже привабливий вигляд. М'ясисті і смачні.</t>
   </si>
   <si>
+    <t>Perets hirkyi</t>
+  </si>
+  <si>
     <t>Перець гіркий</t>
   </si>
   <si>
     <t>catalog/categories/c142.jpg</t>
   </si>
   <si>
+    <t>Kulturnykh sortiv hostroho pertsyu blyzko 3000. Dobre zberihaietsya v sushenomu vyhlyadi.</t>
+  </si>
+  <si>
     <t>Культурних сортів гострого перцю близько 3000. Добре зберігається в сушеному вигляді.</t>
   </si>
   <si>
+    <t>Baklazhany</t>
+  </si>
+  <si>
     <t>Баклажани</t>
   </si>
   <si>
     <t>catalog/categories/c150.jpg</t>
   </si>
   <si>
+    <t>Tsya roslyna stavytysya do rodu paslonovykh i vyroshchuietsya yak odnorichnyk. U izhu vzhyvayut zlehka nedozrili plody tak vony smachnishi.</t>
+  </si>
+  <si>
     <t>Ця рослина ставитися до роду пасльонових і вирощується як однорічник. У їжу вживають злегка недозрілі плоди так вони смачніші.</t>
   </si>
   <si>
+    <t>Tsybulya</t>
+  </si>
+  <si>
     <t>Цибуля</t>
   </si>
   <si>
     <t>catalog/categories/c160.jpg</t>
   </si>
   <si>
+    <t>Riznomanitnist sortiv lukiv ne prypynyaie dyvuvaty: odnorichni, dvorichni i navit bahatorichni. Bahati zelennyu obespechyvat vitaminamy kruhlyi rik.</t>
+  </si>
+  <si>
     <t>Різноманітність сортів луків не припиняє дивувати: однорічні, дворічні і навіть багаторічні. Багаті зеленню обеспечиват вітамінами круглий рік.</t>
   </si>
   <si>
+    <t>Morkva</t>
+  </si>
+  <si>
     <t>Морква</t>
   </si>
   <si>
     <t>catalog/categories/c170.jpg</t>
   </si>
   <si>
+    <t>Morkva mistyt masu korysnykh rechovyn - tse karotyn, soli, kaliyu, pektyny, vitaminy A, V, S, D. Shyroko zastosovuietsya v kulinarii, ne zaminna v dytyachomu kharchuvanni.</t>
+  </si>
+  <si>
     <t>Морква містить масу корисних речовин - це каротин, солі, калію, пектини, вітаміни А, В, С, Д. Широко застосовується в кулінарії, не замінна в дитячому харчуванні.</t>
   </si>
   <si>
+    <t>Buryak</t>
+  </si>
+  <si>
     <t>Буряк</t>
   </si>
   <si>
     <t>catalog/categories/c180.jpg</t>
   </si>
   <si>
+    <t>Buryak maie duzhe vysokymy smakovymy i likuvalnymy vlastyvostyamy, zbahachena iodom, vitaminamy A i V, pokrashchuie obmin rechovyn. U deyakykh sortiv vykorystovuyut i koreneplody i nadzemnu chastynu.</t>
+  </si>
+  <si>
     <t>Буряк має дуже високими смаковими і лікувальними властивостями, збагачена йодом, вітамінами А і В, покращує обмін речовин. У деяких сортів використовують і коренеплоди і надземну частину.</t>
   </si>
   <si>
+    <t>Kavuny</t>
+  </si>
+  <si>
     <t>Кавуни</t>
   </si>
   <si>
     <t>catalog/categories/c190.jpg</t>
   </si>
   <si>
+    <t>Roslyna poshyrylosya z Afryky, proishlo dovhyi selektsiinyi shlyakh. Na sohodni tse - odnorichna steletsya trava z kavalkamy lystyam. Plid kavuna - sokovyta yahoda z bezlichchyu nasinnya.</t>
+  </si>
+  <si>
     <t>Рослина поширилося з Африки, пройшло довгий селекційний шлях. На сьогодні це - однорічна стелеться трава з кавалками листям. Плід кавуна - соковита ягода з безліччю насіння.</t>
   </si>
   <si>
+    <t>Dyni</t>
+  </si>
+  <si>
     <t>Дині</t>
   </si>
   <si>
     <t>catalog/categories/c200.jpg</t>
   </si>
   <si>
+    <t>Tradytsiina bashtannykh kultur dlya stepovoi zony. Holovne daty roslyni bilshe tepla i sontsya. Urozhai, pry dotrymanni ahrotekhniky obrobitku, mozhna otrymaty vzhe v kintsi chervnya.</t>
+  </si>
+  <si>
     <t>Традиційна баштанних культур для степової зони. Головне дати рослині більше тепла і сонця. Урожай, при дотриманні агротехніки обробітку, можна отримати вже в кінці червня.</t>
   </si>
   <si>
+    <t>Harbuzy</t>
+  </si>
+  <si>
     <t>Гарбузи</t>
   </si>
   <si>
     <t>catalog/categories/c210.jpg</t>
   </si>
   <si>
+    <t>Za kilkistyu vmistu zaliza, harbuz - chempion sered ovochiv. Harbuzove nasinnya dzherelo masel, bahatykh mikroelementamy. Yii sokovyta myakot vykorystovuietsya v diietolohii.</t>
+  </si>
+  <si>
     <t>За кількістю вмісту заліза, гарбуз - чемпіон серед овочів. Гарбузове насіння джерело масел, багатих мікроелементами. Її соковита м'якоть використовується в дієтології.</t>
   </si>
   <si>
+    <t>Kabachky</t>
+  </si>
+  <si>
     <t>Кабачки</t>
   </si>
   <si>
     <t>catalog/categories/c220.jpg</t>
   </si>
   <si>
+    <t>Kabachok - tsukini produkt, nyzkokaloriinyi i lehkozasvoyuvanyi orhanizmom, tomu ioho vykorystovuyut v diietolohii i v dytyachomu kharchuvanni.</t>
+  </si>
+  <si>
     <t>Кабачок - цукіні продукт, низькокалорійний і легкозасвоюваний організмом, тому його використовують в дієтології і в дитячому харчуванні.</t>
   </si>
   <si>
+    <t>Patysony</t>
+  </si>
+  <si>
     <t>Патисони</t>
   </si>
   <si>
     <t>catalog/categories/c230.jpg</t>
   </si>
   <si>
+    <t>Plody patysoniv tonkokorye. Myakot bilosnizhna, khrustka i duzhe shchilna. Malyukamy zazvychai pidkhodyat dlya konservatsii, a bilshi plody vykorystovuyut v kulinarii.</t>
+  </si>
+  <si>
     <t>Плоди патисонів тонкокорие. М'якоть білосніжна, хрустка і дуже щільна. Малюками зазвичай підходять для консервації, а більші плоди використовують в кулінарії.</t>
   </si>
   <si>
+    <t>Zeleni kultury</t>
+  </si>
+  <si>
     <t>Зелені культури</t>
   </si>
   <si>
     <t>catalog/categories/c240.jpg</t>
   </si>
   <si>
+    <t>Ranni vitaminy na stolakh - zeleni kultury. Vsi riznovydy salativ, shpynat, shchavel, sparzha, cheremsha.</t>
+  </si>
+  <si>
     <t>Ранні вітаміни на столах - зелені культури. Всі різновиди салатів, шпинат, щавель, спаржа, черемша.</t>
   </si>
   <si>
+    <t>Pryanosmakovi kultury</t>
+  </si>
+  <si>
     <t>Пряносмакові культури</t>
   </si>
   <si>
     <t>catalog/categories/c250.jpg</t>
   </si>
   <si>
+    <t>Do hrupy pryano-smakovykh kultur vkhodyat travy, yaki vykorystovuyutsya yak prypravy: maioran, krip, chaber i bahato-bahato inshykh odnorichnykh i bahatorichnykh roslyn. Vony vidnosno kholodostiiki.</t>
+  </si>
+  <si>
     <t>До групи пряно-смакових культур входять трави, які використовуються як приправи: майоран, кріп, чабер і багато-багато інших однорічних і багаторічних рослин. Вони відносно холодостійкі.</t>
   </si>
   <si>
+    <t>Bobovi kultury</t>
+  </si>
+  <si>
     <t>Бобові культури</t>
   </si>
   <si>
     <t>catalog/categories/c270.jpg</t>
   </si>
   <si>
+    <t>Riznomanitnist vydiv simeistva bobovykh - velychezna. Zastosovuyut ikh yak produkt kharchuvannya.</t>
+  </si>
+  <si>
     <t>Різноманітність видів сімейства бобових - величезна. Застосовують їх як продукт харчування.</t>
   </si>
   <si>
+    <t>Kvasolya</t>
+  </si>
+  <si>
     <t>Квасоля</t>
   </si>
   <si>
     <t>catalog/categories/c280.jpg</t>
   </si>
   <si>
+    <t>Kvasolya vidnosytsya do rozryadu bobovykh z za toho, shcho maie struchkovu formu zapovnenu zernamy i tym ne menshe tse vidminne vid bobovykh roslyna, shcho maie duzhe bahato riznykh sortiv.</t>
+  </si>
+  <si>
     <t>Квасоля відноситься до розряду бобових з за того, що має стручкову форму заповнену зернами і тим не менше це відмінне від бобових рослина, що має дуже багато різних сортів.</t>
   </si>
   <si>
+    <t>Kvasolya sparzheva</t>
+  </si>
+  <si>
     <t>Квасоля спаржева</t>
   </si>
   <si>
     <t>catalog/categories/c281.jpg</t>
   </si>
   <si>
+    <t>Sparzheva kvasolya vyroshchuietsya zarady smachnykh stulok: u nykh vidsutnii perhamentnyi prosharok, tomu kvasolya vzhyvaietsya v izhu tsilkom. Smakom nahaduie sparzhu.</t>
+  </si>
+  <si>
     <t>Спаржева квасоля вирощується заради смачних стулок: у них відсутній пергаментний прошарок, тому квасоля вживається в їжу цілком. Смаком нагадує спаржу.</t>
   </si>
   <si>
+    <t>Kvasolya zernova</t>
+  </si>
+  <si>
     <t>Квасоля зернова</t>
   </si>
   <si>
     <t>catalog/categories/c282.jpg</t>
   </si>
   <si>
+    <t>Lushchylni sorty kvasoli vyroshchuyutsya vyklyuchno dlya vzhyvannya v izhu zeren: duzhe pozhyvnykh i mistyat velyku kilkist bilka.</t>
+  </si>
+  <si>
     <t>Лущильні сорти квасолі вирощуються виключно для вживання в їжу зерен: дуже поживних і містять велику кількість білка.</t>
   </si>
   <si>
+    <t>Kukurudza</t>
+  </si>
+  <si>
     <t>Кукурудза</t>
   </si>
   <si>
     <t>catalog/categories/c290.jpg</t>
   </si>
   <si>
+    <t>Kukurudza - tsarytsya poliv, tse odnorichna travyanysta roslyna vidnosytsya do zlakovykh kultur.</t>
+  </si>
+  <si>
     <t>Кукурудза - цариця полів, це однорічна трав'яниста рослина відноситься до злакових культур.</t>
   </si>
   <si>
+    <t>Kvity</t>
+  </si>
+  <si>
     <t>Квіти</t>
   </si>
   <si>
     <t>catalog/categories/c330.jpg</t>
   </si>
   <si>
+    <t>Aromaty, riznomanitnist koloru, nizhnist, trepet i lyubov - vse tse vidnosytsya do bahatotysyachnoi armii kvitiv vsikh vydiv, vsikh katehorii i vsikh natsionalnostei.</t>
+  </si>
+  <si>
     <t>Аромати, різноманітність кольору, ніжність, трепет і любов - все це відноситься до багатотисячної армії квітів всіх видів, всіх категорій і всіх національностей.</t>
   </si>
   <si>
+    <t>Kvity odnorichni</t>
+  </si>
+  <si>
     <t>Квіти однорічні</t>
   </si>
   <si>
     <t>catalog/categories/c331.jpg</t>
   </si>
   <si>
+    <t>Velykyi diapazon koloriv, bahatyi vybir form, riznytsya terminiv tsvitinnya - daie mozhlyvist stvoryuvaty bud-yaki kompozytsii. I te, shcho roslyny odnorichni - dozvolyaie eksperymentuvaty neskinchenno.</t>
+  </si>
+  <si>
     <t>Великий діапазон кольорів, багатий вибір форм, різниця термінів цвітіння - дає можливість створювати будь-які композиції. І те, що рослини однорічні - дозволяє експериментувати нескінченно.</t>
   </si>
   <si>
+    <t>Kvity bahatorichni</t>
+  </si>
+  <si>
     <t>Квіти багаторічні</t>
   </si>
   <si>
     <t>catalog/categories/c332.jpg</t>
   </si>
   <si>
+    <t>Bahatorichnyky zazvychai dayut mozhlyvist formuvaty kompozytsii na kilka rokiv vpered. Prekrasno susidyat zi svoimy pobratymamy i ne vybahlyvi do gruntu. Tse i vysokorosli, i tsybulynni (typu muskary abo ptytsemlechnyk), i stelyashchyesya pochvopokryvni roslyny.</t>
+  </si>
+  <si>
     <t>Багаторічники зазвичай дають можливість формувати композиції на кілька років вперед. Прекрасно сусідять зі своїми побратимами і не вибагливі до ґрунту. Це і високорослі, і цибулинні (типу мускари або птицемлечник), і стелящиеся почвопокривні рослини.</t>
   </si>
   <si>
+    <t>Dobryva ta zakhyst</t>
+  </si>
+  <si>
     <t>Добрива та захист</t>
   </si>
   <si>
     <t>catalog/categories/c400.jpg</t>
   </si>
   <si>
+    <t>Herbitsydy</t>
+  </si>
+  <si>
     <t>Гербіциди</t>
   </si>
   <si>
     <t>catalog/categories/c401.jpg</t>
   </si>
   <si>
+    <t>Insektytsydy</t>
+  </si>
+  <si>
     <t>Інсектициди</t>
   </si>
   <si>
     <t>catalog/categories/c402.jpg</t>
   </si>
   <si>
+    <t>Funhitsydy</t>
+  </si>
+  <si>
     <t>Фунгіциди</t>
   </si>
   <si>
     <t>catalog/categories/c403.jpg</t>
   </si>
   <si>
+    <t>Biopreparaty</t>
+  </si>
+  <si>
     <t>Біопрепарати</t>
   </si>
   <si>
     <t>catalog/categories/c405.jpg</t>
   </si>
   <si>
+    <t>Prylypachi</t>
+  </si>
+  <si>
     <t>Прилипачі</t>
   </si>
   <si>
     <t>catalog/categories/c406.jpg</t>
   </si>
   <si>
+    <t>Dobryva ta stymulyatory</t>
+  </si>
+  <si>
     <t>Добрива та стимулятори</t>
   </si>
   <si>
     <t>catalog/categories/c407.jpg</t>
   </si>
   <si>
+    <t>Suputni tovary</t>
+  </si>
+  <si>
     <t>Супутні товари</t>
   </si>
   <si>
@@ -403,6 +640,9 @@
   </si>
   <si>
     <t>keyword(en-gb)</t>
+  </si>
+  <si>
+    <t>keyword(uk-ua)</t>
   </si>
   <si>
     <t>tomati</t>
@@ -858,10 +1098,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:Q42"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:17">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -898,8 +1138,23 @@
       <c r="L1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12">
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17">
       <c r="A2">
         <v>100</v>
       </c>
@@ -907,33 +1162,46 @@
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2">
+        <v>17</v>
+      </c>
+      <c r="D2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2">
         <v>1</v>
       </c>
-      <c r="E2" t="s">
-        <v>13</v>
-      </c>
       <c r="F2" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="G2" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2"/>
-      <c r="J2">
-        <v>0</v>
-      </c>
-      <c r="K2"/>
+        <v>21</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" t="s">
+        <v>20</v>
+      </c>
       <c r="L2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+        <v>21</v>
+      </c>
+      <c r="M2"/>
+      <c r="N2"/>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2"/>
+      <c r="Q2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17">
       <c r="A3">
         <v>101</v>
       </c>
@@ -941,33 +1209,46 @@
         <v>100</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3">
         <v>2</v>
       </c>
-      <c r="E3" t="s">
-        <v>17</v>
-      </c>
       <c r="F3" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="G3" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="H3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I3"/>
-      <c r="J3">
-        <v>0</v>
-      </c>
-      <c r="K3"/>
+        <v>27</v>
+      </c>
+      <c r="I3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" t="s">
+        <v>26</v>
+      </c>
       <c r="L3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
+        <v>27</v>
+      </c>
+      <c r="M3"/>
+      <c r="N3"/>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3"/>
+      <c r="Q3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17">
       <c r="A4">
         <v>102</v>
       </c>
@@ -975,33 +1256,46 @@
         <v>100</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4">
+        <v>28</v>
+      </c>
+      <c r="D4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4">
         <v>3</v>
       </c>
-      <c r="E4" t="s">
-        <v>20</v>
-      </c>
       <c r="F4" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="H4" t="s">
-        <v>21</v>
-      </c>
-      <c r="I4"/>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4"/>
+        <v>32</v>
+      </c>
+      <c r="I4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" t="s">
+        <v>29</v>
+      </c>
+      <c r="K4" t="s">
+        <v>31</v>
+      </c>
       <c r="L4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
+        <v>32</v>
+      </c>
+      <c r="M4"/>
+      <c r="N4"/>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4"/>
+      <c r="Q4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17">
       <c r="A5">
         <v>103</v>
       </c>
@@ -1009,33 +1303,46 @@
         <v>100</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5">
+        <v>33</v>
+      </c>
+      <c r="D5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5">
         <v>4</v>
       </c>
-      <c r="E5" t="s">
-        <v>23</v>
-      </c>
       <c r="F5" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="G5" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="H5" t="s">
-        <v>24</v>
-      </c>
-      <c r="I5"/>
-      <c r="J5">
-        <v>0</v>
-      </c>
-      <c r="K5"/>
+        <v>37</v>
+      </c>
+      <c r="I5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K5" t="s">
+        <v>36</v>
+      </c>
       <c r="L5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
+        <v>37</v>
+      </c>
+      <c r="M5"/>
+      <c r="N5"/>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5"/>
+      <c r="Q5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17">
       <c r="A6">
         <v>110</v>
       </c>
@@ -1043,33 +1350,46 @@
         <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6">
+        <v>38</v>
+      </c>
+      <c r="D6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6">
         <v>5</v>
       </c>
-      <c r="E6" t="s">
-        <v>26</v>
-      </c>
       <c r="F6" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="G6" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="H6" t="s">
-        <v>27</v>
-      </c>
-      <c r="I6"/>
-      <c r="J6">
-        <v>0</v>
-      </c>
-      <c r="K6"/>
+        <v>42</v>
+      </c>
+      <c r="I6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J6" t="s">
+        <v>39</v>
+      </c>
+      <c r="K6" t="s">
+        <v>41</v>
+      </c>
       <c r="L6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
+        <v>42</v>
+      </c>
+      <c r="M6"/>
+      <c r="N6"/>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6"/>
+      <c r="Q6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17">
       <c r="A7">
         <v>120</v>
       </c>
@@ -1077,33 +1397,46 @@
         <v>0</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7">
+        <v>43</v>
+      </c>
+      <c r="D7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7">
         <v>6</v>
       </c>
-      <c r="E7" t="s">
-        <v>29</v>
-      </c>
       <c r="F7" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="G7" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="H7" t="s">
-        <v>30</v>
-      </c>
-      <c r="I7"/>
-      <c r="J7">
-        <v>0</v>
-      </c>
-      <c r="K7"/>
+        <v>47</v>
+      </c>
+      <c r="I7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J7" t="s">
+        <v>44</v>
+      </c>
+      <c r="K7" t="s">
+        <v>46</v>
+      </c>
       <c r="L7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
+        <v>47</v>
+      </c>
+      <c r="M7"/>
+      <c r="N7"/>
+      <c r="O7">
+        <v>0</v>
+      </c>
+      <c r="P7"/>
+      <c r="Q7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17">
       <c r="A8">
         <v>121</v>
       </c>
@@ -1111,33 +1444,46 @@
         <v>120</v>
       </c>
       <c r="C8" t="s">
-        <v>31</v>
-      </c>
-      <c r="D8">
+        <v>48</v>
+      </c>
+      <c r="D8" t="s">
+        <v>49</v>
+      </c>
+      <c r="E8">
         <v>7</v>
       </c>
-      <c r="E8" t="s">
-        <v>32</v>
-      </c>
       <c r="F8" t="s">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="G8" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="H8" t="s">
-        <v>33</v>
-      </c>
-      <c r="I8"/>
-      <c r="J8">
-        <v>0</v>
-      </c>
-      <c r="K8"/>
+        <v>52</v>
+      </c>
+      <c r="I8" t="s">
+        <v>48</v>
+      </c>
+      <c r="J8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K8" t="s">
+        <v>51</v>
+      </c>
       <c r="L8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
+        <v>52</v>
+      </c>
+      <c r="M8"/>
+      <c r="N8"/>
+      <c r="O8">
+        <v>0</v>
+      </c>
+      <c r="P8"/>
+      <c r="Q8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17">
       <c r="A9">
         <v>122</v>
       </c>
@@ -1145,33 +1491,46 @@
         <v>120</v>
       </c>
       <c r="C9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9">
+        <v>53</v>
+      </c>
+      <c r="D9" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9">
         <v>8</v>
       </c>
-      <c r="E9" t="s">
-        <v>35</v>
-      </c>
       <c r="F9" t="s">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="G9" t="s">
-        <v>34</v>
+        <v>56</v>
       </c>
       <c r="H9" t="s">
-        <v>36</v>
-      </c>
-      <c r="I9"/>
-      <c r="J9">
-        <v>0</v>
-      </c>
-      <c r="K9"/>
+        <v>57</v>
+      </c>
+      <c r="I9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K9" t="s">
+        <v>56</v>
+      </c>
       <c r="L9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
+        <v>57</v>
+      </c>
+      <c r="M9"/>
+      <c r="N9"/>
+      <c r="O9">
+        <v>0</v>
+      </c>
+      <c r="P9"/>
+      <c r="Q9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17">
       <c r="A10">
         <v>123</v>
       </c>
@@ -1179,33 +1538,46 @@
         <v>120</v>
       </c>
       <c r="C10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10">
+        <v>58</v>
+      </c>
+      <c r="D10" t="s">
+        <v>59</v>
+      </c>
+      <c r="E10">
         <v>9</v>
       </c>
-      <c r="E10" t="s">
-        <v>38</v>
-      </c>
       <c r="F10" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="G10" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="H10" t="s">
-        <v>39</v>
-      </c>
-      <c r="I10"/>
-      <c r="J10">
-        <v>0</v>
-      </c>
-      <c r="K10"/>
+        <v>62</v>
+      </c>
+      <c r="I10" t="s">
+        <v>58</v>
+      </c>
+      <c r="J10" t="s">
+        <v>59</v>
+      </c>
+      <c r="K10" t="s">
+        <v>61</v>
+      </c>
       <c r="L10" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12">
+        <v>62</v>
+      </c>
+      <c r="M10"/>
+      <c r="N10"/>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="P10"/>
+      <c r="Q10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17">
       <c r="A11">
         <v>124</v>
       </c>
@@ -1213,31 +1585,44 @@
         <v>120</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D11">
+        <v>63</v>
+      </c>
+      <c r="D11" t="s">
+        <v>64</v>
+      </c>
+      <c r="E11">
         <v>10</v>
       </c>
-      <c r="E11"/>
-      <c r="F11" t="s">
-        <v>41</v>
-      </c>
+      <c r="F11"/>
       <c r="G11" t="s">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="H11" t="s">
-        <v>41</v>
-      </c>
-      <c r="I11"/>
-      <c r="J11">
-        <v>0</v>
-      </c>
-      <c r="K11"/>
+        <v>66</v>
+      </c>
+      <c r="I11" t="s">
+        <v>63</v>
+      </c>
+      <c r="J11" t="s">
+        <v>64</v>
+      </c>
+      <c r="K11" t="s">
+        <v>65</v>
+      </c>
       <c r="L11" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12">
+        <v>66</v>
+      </c>
+      <c r="M11"/>
+      <c r="N11"/>
+      <c r="O11">
+        <v>0</v>
+      </c>
+      <c r="P11"/>
+      <c r="Q11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17">
       <c r="A12">
         <v>130</v>
       </c>
@@ -1245,33 +1630,46 @@
         <v>0</v>
       </c>
       <c r="C12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12">
+        <v>67</v>
+      </c>
+      <c r="D12" t="s">
+        <v>68</v>
+      </c>
+      <c r="E12">
         <v>11</v>
       </c>
-      <c r="E12" t="s">
-        <v>43</v>
-      </c>
       <c r="F12" t="s">
-        <v>44</v>
+        <v>69</v>
       </c>
       <c r="G12" t="s">
-        <v>42</v>
+        <v>70</v>
       </c>
       <c r="H12" t="s">
-        <v>44</v>
-      </c>
-      <c r="I12"/>
-      <c r="J12">
-        <v>0</v>
-      </c>
-      <c r="K12"/>
+        <v>71</v>
+      </c>
+      <c r="I12" t="s">
+        <v>67</v>
+      </c>
+      <c r="J12" t="s">
+        <v>68</v>
+      </c>
+      <c r="K12" t="s">
+        <v>70</v>
+      </c>
       <c r="L12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12">
+        <v>71</v>
+      </c>
+      <c r="M12"/>
+      <c r="N12"/>
+      <c r="O12">
+        <v>0</v>
+      </c>
+      <c r="P12"/>
+      <c r="Q12" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17">
       <c r="A13">
         <v>140</v>
       </c>
@@ -1279,33 +1677,46 @@
         <v>0</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
-      </c>
-      <c r="D13">
+        <v>72</v>
+      </c>
+      <c r="D13" t="s">
+        <v>73</v>
+      </c>
+      <c r="E13">
         <v>12</v>
       </c>
-      <c r="E13" t="s">
-        <v>46</v>
-      </c>
       <c r="F13" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="G13" t="s">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="H13" t="s">
-        <v>47</v>
-      </c>
-      <c r="I13"/>
-      <c r="J13">
-        <v>0</v>
-      </c>
-      <c r="K13"/>
+        <v>76</v>
+      </c>
+      <c r="I13" t="s">
+        <v>72</v>
+      </c>
+      <c r="J13" t="s">
+        <v>73</v>
+      </c>
+      <c r="K13" t="s">
+        <v>75</v>
+      </c>
       <c r="L13" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12">
+        <v>76</v>
+      </c>
+      <c r="M13"/>
+      <c r="N13"/>
+      <c r="O13">
+        <v>0</v>
+      </c>
+      <c r="P13"/>
+      <c r="Q13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17">
       <c r="A14">
         <v>141</v>
       </c>
@@ -1313,33 +1724,46 @@
         <v>140</v>
       </c>
       <c r="C14" t="s">
-        <v>48</v>
-      </c>
-      <c r="D14">
+        <v>77</v>
+      </c>
+      <c r="D14" t="s">
+        <v>78</v>
+      </c>
+      <c r="E14">
         <v>13</v>
       </c>
-      <c r="E14" t="s">
-        <v>49</v>
-      </c>
       <c r="F14" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
       <c r="G14" t="s">
-        <v>48</v>
+        <v>80</v>
       </c>
       <c r="H14" t="s">
-        <v>50</v>
-      </c>
-      <c r="I14"/>
-      <c r="J14">
-        <v>0</v>
-      </c>
-      <c r="K14"/>
+        <v>81</v>
+      </c>
+      <c r="I14" t="s">
+        <v>77</v>
+      </c>
+      <c r="J14" t="s">
+        <v>78</v>
+      </c>
+      <c r="K14" t="s">
+        <v>80</v>
+      </c>
       <c r="L14" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12">
+        <v>81</v>
+      </c>
+      <c r="M14"/>
+      <c r="N14"/>
+      <c r="O14">
+        <v>0</v>
+      </c>
+      <c r="P14"/>
+      <c r="Q14" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17">
       <c r="A15">
         <v>142</v>
       </c>
@@ -1347,33 +1771,46 @@
         <v>140</v>
       </c>
       <c r="C15" t="s">
-        <v>51</v>
-      </c>
-      <c r="D15">
+        <v>82</v>
+      </c>
+      <c r="D15" t="s">
+        <v>83</v>
+      </c>
+      <c r="E15">
         <v>14</v>
       </c>
-      <c r="E15" t="s">
-        <v>52</v>
-      </c>
       <c r="F15" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="G15" t="s">
-        <v>51</v>
+        <v>85</v>
       </c>
       <c r="H15" t="s">
-        <v>53</v>
-      </c>
-      <c r="I15"/>
-      <c r="J15">
-        <v>0</v>
-      </c>
-      <c r="K15"/>
+        <v>86</v>
+      </c>
+      <c r="I15" t="s">
+        <v>82</v>
+      </c>
+      <c r="J15" t="s">
+        <v>83</v>
+      </c>
+      <c r="K15" t="s">
+        <v>85</v>
+      </c>
       <c r="L15" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12">
+        <v>86</v>
+      </c>
+      <c r="M15"/>
+      <c r="N15"/>
+      <c r="O15">
+        <v>0</v>
+      </c>
+      <c r="P15"/>
+      <c r="Q15" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17">
       <c r="A16">
         <v>150</v>
       </c>
@@ -1381,33 +1818,46 @@
         <v>0</v>
       </c>
       <c r="C16" t="s">
-        <v>54</v>
-      </c>
-      <c r="D16">
+        <v>87</v>
+      </c>
+      <c r="D16" t="s">
+        <v>88</v>
+      </c>
+      <c r="E16">
         <v>15</v>
       </c>
-      <c r="E16" t="s">
-        <v>55</v>
-      </c>
       <c r="F16" t="s">
-        <v>56</v>
+        <v>89</v>
       </c>
       <c r="G16" t="s">
-        <v>54</v>
+        <v>90</v>
       </c>
       <c r="H16" t="s">
-        <v>56</v>
-      </c>
-      <c r="I16"/>
-      <c r="J16">
-        <v>0</v>
-      </c>
-      <c r="K16"/>
+        <v>91</v>
+      </c>
+      <c r="I16" t="s">
+        <v>87</v>
+      </c>
+      <c r="J16" t="s">
+        <v>88</v>
+      </c>
+      <c r="K16" t="s">
+        <v>90</v>
+      </c>
       <c r="L16" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12">
+        <v>91</v>
+      </c>
+      <c r="M16"/>
+      <c r="N16"/>
+      <c r="O16">
+        <v>0</v>
+      </c>
+      <c r="P16"/>
+      <c r="Q16" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17">
       <c r="A17">
         <v>160</v>
       </c>
@@ -1415,33 +1865,46 @@
         <v>0</v>
       </c>
       <c r="C17" t="s">
-        <v>57</v>
-      </c>
-      <c r="D17">
+        <v>92</v>
+      </c>
+      <c r="D17" t="s">
+        <v>93</v>
+      </c>
+      <c r="E17">
         <v>16</v>
       </c>
-      <c r="E17" t="s">
-        <v>58</v>
-      </c>
       <c r="F17" t="s">
-        <v>59</v>
+        <v>94</v>
       </c>
       <c r="G17" t="s">
-        <v>57</v>
+        <v>95</v>
       </c>
       <c r="H17" t="s">
-        <v>59</v>
-      </c>
-      <c r="I17"/>
-      <c r="J17">
-        <v>0</v>
-      </c>
-      <c r="K17"/>
+        <v>96</v>
+      </c>
+      <c r="I17" t="s">
+        <v>92</v>
+      </c>
+      <c r="J17" t="s">
+        <v>93</v>
+      </c>
+      <c r="K17" t="s">
+        <v>95</v>
+      </c>
       <c r="L17" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12">
+        <v>96</v>
+      </c>
+      <c r="M17"/>
+      <c r="N17"/>
+      <c r="O17">
+        <v>0</v>
+      </c>
+      <c r="P17"/>
+      <c r="Q17" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17">
       <c r="A18">
         <v>170</v>
       </c>
@@ -1449,33 +1912,46 @@
         <v>0</v>
       </c>
       <c r="C18" t="s">
-        <v>60</v>
-      </c>
-      <c r="D18">
+        <v>97</v>
+      </c>
+      <c r="D18" t="s">
+        <v>98</v>
+      </c>
+      <c r="E18">
         <v>17</v>
       </c>
-      <c r="E18" t="s">
-        <v>61</v>
-      </c>
       <c r="F18" t="s">
-        <v>62</v>
+        <v>99</v>
       </c>
       <c r="G18" t="s">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="H18" t="s">
-        <v>62</v>
-      </c>
-      <c r="I18"/>
-      <c r="J18">
-        <v>0</v>
-      </c>
-      <c r="K18"/>
+        <v>101</v>
+      </c>
+      <c r="I18" t="s">
+        <v>97</v>
+      </c>
+      <c r="J18" t="s">
+        <v>98</v>
+      </c>
+      <c r="K18" t="s">
+        <v>100</v>
+      </c>
       <c r="L18" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12">
+        <v>101</v>
+      </c>
+      <c r="M18"/>
+      <c r="N18"/>
+      <c r="O18">
+        <v>0</v>
+      </c>
+      <c r="P18"/>
+      <c r="Q18" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17">
       <c r="A19">
         <v>180</v>
       </c>
@@ -1483,33 +1959,46 @@
         <v>0</v>
       </c>
       <c r="C19" t="s">
-        <v>63</v>
-      </c>
-      <c r="D19">
+        <v>102</v>
+      </c>
+      <c r="D19" t="s">
+        <v>103</v>
+      </c>
+      <c r="E19">
         <v>18</v>
       </c>
-      <c r="E19" t="s">
-        <v>64</v>
-      </c>
       <c r="F19" t="s">
-        <v>65</v>
+        <v>104</v>
       </c>
       <c r="G19" t="s">
-        <v>63</v>
+        <v>105</v>
       </c>
       <c r="H19" t="s">
-        <v>65</v>
-      </c>
-      <c r="I19"/>
-      <c r="J19">
-        <v>0</v>
-      </c>
-      <c r="K19"/>
+        <v>106</v>
+      </c>
+      <c r="I19" t="s">
+        <v>102</v>
+      </c>
+      <c r="J19" t="s">
+        <v>103</v>
+      </c>
+      <c r="K19" t="s">
+        <v>105</v>
+      </c>
       <c r="L19" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12">
+        <v>106</v>
+      </c>
+      <c r="M19"/>
+      <c r="N19"/>
+      <c r="O19">
+        <v>0</v>
+      </c>
+      <c r="P19"/>
+      <c r="Q19" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17">
       <c r="A20">
         <v>190</v>
       </c>
@@ -1517,33 +2006,46 @@
         <v>0</v>
       </c>
       <c r="C20" t="s">
-        <v>66</v>
-      </c>
-      <c r="D20">
+        <v>107</v>
+      </c>
+      <c r="D20" t="s">
+        <v>108</v>
+      </c>
+      <c r="E20">
         <v>19</v>
       </c>
-      <c r="E20" t="s">
-        <v>67</v>
-      </c>
       <c r="F20" t="s">
-        <v>68</v>
+        <v>109</v>
       </c>
       <c r="G20" t="s">
-        <v>66</v>
+        <v>110</v>
       </c>
       <c r="H20" t="s">
-        <v>68</v>
-      </c>
-      <c r="I20"/>
-      <c r="J20">
-        <v>0</v>
-      </c>
-      <c r="K20"/>
+        <v>111</v>
+      </c>
+      <c r="I20" t="s">
+        <v>107</v>
+      </c>
+      <c r="J20" t="s">
+        <v>108</v>
+      </c>
+      <c r="K20" t="s">
+        <v>110</v>
+      </c>
       <c r="L20" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12">
+        <v>111</v>
+      </c>
+      <c r="M20"/>
+      <c r="N20"/>
+      <c r="O20">
+        <v>0</v>
+      </c>
+      <c r="P20"/>
+      <c r="Q20" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17">
       <c r="A21">
         <v>200</v>
       </c>
@@ -1551,33 +2053,46 @@
         <v>0</v>
       </c>
       <c r="C21" t="s">
-        <v>69</v>
-      </c>
-      <c r="D21">
+        <v>112</v>
+      </c>
+      <c r="D21" t="s">
+        <v>113</v>
+      </c>
+      <c r="E21">
         <v>20</v>
       </c>
-      <c r="E21" t="s">
-        <v>70</v>
-      </c>
       <c r="F21" t="s">
-        <v>71</v>
+        <v>114</v>
       </c>
       <c r="G21" t="s">
-        <v>69</v>
+        <v>115</v>
       </c>
       <c r="H21" t="s">
-        <v>71</v>
-      </c>
-      <c r="I21"/>
-      <c r="J21">
-        <v>0</v>
-      </c>
-      <c r="K21"/>
+        <v>116</v>
+      </c>
+      <c r="I21" t="s">
+        <v>112</v>
+      </c>
+      <c r="J21" t="s">
+        <v>113</v>
+      </c>
+      <c r="K21" t="s">
+        <v>115</v>
+      </c>
       <c r="L21" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12">
+        <v>116</v>
+      </c>
+      <c r="M21"/>
+      <c r="N21"/>
+      <c r="O21">
+        <v>0</v>
+      </c>
+      <c r="P21"/>
+      <c r="Q21" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17">
       <c r="A22">
         <v>210</v>
       </c>
@@ -1585,33 +2100,46 @@
         <v>0</v>
       </c>
       <c r="C22" t="s">
-        <v>72</v>
-      </c>
-      <c r="D22">
+        <v>117</v>
+      </c>
+      <c r="D22" t="s">
+        <v>118</v>
+      </c>
+      <c r="E22">
         <v>21</v>
       </c>
-      <c r="E22" t="s">
-        <v>73</v>
-      </c>
       <c r="F22" t="s">
-        <v>74</v>
+        <v>119</v>
       </c>
       <c r="G22" t="s">
-        <v>72</v>
+        <v>120</v>
       </c>
       <c r="H22" t="s">
-        <v>74</v>
-      </c>
-      <c r="I22"/>
-      <c r="J22">
-        <v>0</v>
-      </c>
-      <c r="K22"/>
+        <v>121</v>
+      </c>
+      <c r="I22" t="s">
+        <v>117</v>
+      </c>
+      <c r="J22" t="s">
+        <v>118</v>
+      </c>
+      <c r="K22" t="s">
+        <v>120</v>
+      </c>
       <c r="L22" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12">
+        <v>121</v>
+      </c>
+      <c r="M22"/>
+      <c r="N22"/>
+      <c r="O22">
+        <v>0</v>
+      </c>
+      <c r="P22"/>
+      <c r="Q22" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17">
       <c r="A23">
         <v>220</v>
       </c>
@@ -1619,33 +2147,46 @@
         <v>0</v>
       </c>
       <c r="C23" t="s">
-        <v>75</v>
-      </c>
-      <c r="D23">
-        <v>22</v>
-      </c>
-      <c r="E23" t="s">
-        <v>76</v>
+        <v>122</v>
+      </c>
+      <c r="D23" t="s">
+        <v>123</v>
+      </c>
+      <c r="E23">
+        <v>22</v>
       </c>
       <c r="F23" t="s">
-        <v>77</v>
+        <v>124</v>
       </c>
       <c r="G23" t="s">
-        <v>75</v>
+        <v>125</v>
       </c>
       <c r="H23" t="s">
-        <v>77</v>
-      </c>
-      <c r="I23"/>
-      <c r="J23">
-        <v>0</v>
-      </c>
-      <c r="K23"/>
+        <v>126</v>
+      </c>
+      <c r="I23" t="s">
+        <v>122</v>
+      </c>
+      <c r="J23" t="s">
+        <v>123</v>
+      </c>
+      <c r="K23" t="s">
+        <v>125</v>
+      </c>
       <c r="L23" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12">
+        <v>126</v>
+      </c>
+      <c r="M23"/>
+      <c r="N23"/>
+      <c r="O23">
+        <v>0</v>
+      </c>
+      <c r="P23"/>
+      <c r="Q23" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17">
       <c r="A24">
         <v>230</v>
       </c>
@@ -1653,33 +2194,46 @@
         <v>0</v>
       </c>
       <c r="C24" t="s">
-        <v>78</v>
-      </c>
-      <c r="D24">
+        <v>127</v>
+      </c>
+      <c r="D24" t="s">
+        <v>128</v>
+      </c>
+      <c r="E24">
         <v>23</v>
       </c>
-      <c r="E24" t="s">
-        <v>79</v>
-      </c>
       <c r="F24" t="s">
-        <v>80</v>
+        <v>129</v>
       </c>
       <c r="G24" t="s">
-        <v>78</v>
+        <v>130</v>
       </c>
       <c r="H24" t="s">
-        <v>80</v>
-      </c>
-      <c r="I24"/>
-      <c r="J24">
-        <v>0</v>
-      </c>
-      <c r="K24"/>
+        <v>131</v>
+      </c>
+      <c r="I24" t="s">
+        <v>127</v>
+      </c>
+      <c r="J24" t="s">
+        <v>128</v>
+      </c>
+      <c r="K24" t="s">
+        <v>130</v>
+      </c>
       <c r="L24" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12">
+        <v>131</v>
+      </c>
+      <c r="M24"/>
+      <c r="N24"/>
+      <c r="O24">
+        <v>0</v>
+      </c>
+      <c r="P24"/>
+      <c r="Q24" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17">
       <c r="A25">
         <v>240</v>
       </c>
@@ -1687,33 +2241,46 @@
         <v>0</v>
       </c>
       <c r="C25" t="s">
-        <v>81</v>
-      </c>
-      <c r="D25">
+        <v>132</v>
+      </c>
+      <c r="D25" t="s">
+        <v>133</v>
+      </c>
+      <c r="E25">
         <v>24</v>
       </c>
-      <c r="E25" t="s">
-        <v>82</v>
-      </c>
       <c r="F25" t="s">
-        <v>83</v>
+        <v>134</v>
       </c>
       <c r="G25" t="s">
-        <v>81</v>
+        <v>135</v>
       </c>
       <c r="H25" t="s">
-        <v>83</v>
-      </c>
-      <c r="I25"/>
-      <c r="J25">
-        <v>0</v>
-      </c>
-      <c r="K25"/>
+        <v>136</v>
+      </c>
+      <c r="I25" t="s">
+        <v>132</v>
+      </c>
+      <c r="J25" t="s">
+        <v>133</v>
+      </c>
+      <c r="K25" t="s">
+        <v>135</v>
+      </c>
       <c r="L25" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12">
+        <v>136</v>
+      </c>
+      <c r="M25"/>
+      <c r="N25"/>
+      <c r="O25">
+        <v>0</v>
+      </c>
+      <c r="P25"/>
+      <c r="Q25" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17">
       <c r="A26">
         <v>250</v>
       </c>
@@ -1721,33 +2288,46 @@
         <v>0</v>
       </c>
       <c r="C26" t="s">
-        <v>84</v>
-      </c>
-      <c r="D26">
+        <v>137</v>
+      </c>
+      <c r="D26" t="s">
+        <v>138</v>
+      </c>
+      <c r="E26">
         <v>25</v>
       </c>
-      <c r="E26" t="s">
-        <v>85</v>
-      </c>
       <c r="F26" t="s">
-        <v>86</v>
+        <v>139</v>
       </c>
       <c r="G26" t="s">
-        <v>84</v>
+        <v>140</v>
       </c>
       <c r="H26" t="s">
-        <v>86</v>
-      </c>
-      <c r="I26"/>
-      <c r="J26">
-        <v>0</v>
-      </c>
-      <c r="K26"/>
+        <v>141</v>
+      </c>
+      <c r="I26" t="s">
+        <v>137</v>
+      </c>
+      <c r="J26" t="s">
+        <v>138</v>
+      </c>
+      <c r="K26" t="s">
+        <v>140</v>
+      </c>
       <c r="L26" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12">
+        <v>141</v>
+      </c>
+      <c r="M26"/>
+      <c r="N26"/>
+      <c r="O26">
+        <v>0</v>
+      </c>
+      <c r="P26"/>
+      <c r="Q26" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17">
       <c r="A27">
         <v>270</v>
       </c>
@@ -1755,33 +2335,46 @@
         <v>0</v>
       </c>
       <c r="C27" t="s">
-        <v>87</v>
-      </c>
-      <c r="D27">
+        <v>142</v>
+      </c>
+      <c r="D27" t="s">
+        <v>143</v>
+      </c>
+      <c r="E27">
         <v>26</v>
       </c>
-      <c r="E27" t="s">
-        <v>88</v>
-      </c>
       <c r="F27" t="s">
-        <v>89</v>
+        <v>144</v>
       </c>
       <c r="G27" t="s">
-        <v>87</v>
+        <v>145</v>
       </c>
       <c r="H27" t="s">
-        <v>89</v>
-      </c>
-      <c r="I27"/>
-      <c r="J27">
-        <v>0</v>
-      </c>
-      <c r="K27"/>
+        <v>146</v>
+      </c>
+      <c r="I27" t="s">
+        <v>142</v>
+      </c>
+      <c r="J27" t="s">
+        <v>143</v>
+      </c>
+      <c r="K27" t="s">
+        <v>145</v>
+      </c>
       <c r="L27" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12">
+        <v>146</v>
+      </c>
+      <c r="M27"/>
+      <c r="N27"/>
+      <c r="O27">
+        <v>0</v>
+      </c>
+      <c r="P27"/>
+      <c r="Q27" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17">
       <c r="A28">
         <v>280</v>
       </c>
@@ -1789,33 +2382,46 @@
         <v>0</v>
       </c>
       <c r="C28" t="s">
-        <v>90</v>
-      </c>
-      <c r="D28">
+        <v>147</v>
+      </c>
+      <c r="D28" t="s">
+        <v>148</v>
+      </c>
+      <c r="E28">
         <v>27</v>
       </c>
-      <c r="E28" t="s">
-        <v>91</v>
-      </c>
       <c r="F28" t="s">
-        <v>92</v>
+        <v>149</v>
       </c>
       <c r="G28" t="s">
-        <v>90</v>
+        <v>150</v>
       </c>
       <c r="H28" t="s">
-        <v>92</v>
-      </c>
-      <c r="I28"/>
-      <c r="J28">
-        <v>0</v>
-      </c>
-      <c r="K28"/>
+        <v>151</v>
+      </c>
+      <c r="I28" t="s">
+        <v>147</v>
+      </c>
+      <c r="J28" t="s">
+        <v>148</v>
+      </c>
+      <c r="K28" t="s">
+        <v>150</v>
+      </c>
       <c r="L28" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12">
+        <v>151</v>
+      </c>
+      <c r="M28"/>
+      <c r="N28"/>
+      <c r="O28">
+        <v>0</v>
+      </c>
+      <c r="P28"/>
+      <c r="Q28" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17">
       <c r="A29">
         <v>281</v>
       </c>
@@ -1823,33 +2429,46 @@
         <v>280</v>
       </c>
       <c r="C29" t="s">
-        <v>93</v>
-      </c>
-      <c r="D29">
+        <v>152</v>
+      </c>
+      <c r="D29" t="s">
+        <v>153</v>
+      </c>
+      <c r="E29">
         <v>28</v>
       </c>
-      <c r="E29" t="s">
-        <v>94</v>
-      </c>
       <c r="F29" t="s">
-        <v>95</v>
+        <v>154</v>
       </c>
       <c r="G29" t="s">
-        <v>93</v>
+        <v>155</v>
       </c>
       <c r="H29" t="s">
-        <v>95</v>
-      </c>
-      <c r="I29"/>
-      <c r="J29">
-        <v>0</v>
-      </c>
-      <c r="K29"/>
+        <v>156</v>
+      </c>
+      <c r="I29" t="s">
+        <v>152</v>
+      </c>
+      <c r="J29" t="s">
+        <v>153</v>
+      </c>
+      <c r="K29" t="s">
+        <v>155</v>
+      </c>
       <c r="L29" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12">
+        <v>156</v>
+      </c>
+      <c r="M29"/>
+      <c r="N29"/>
+      <c r="O29">
+        <v>0</v>
+      </c>
+      <c r="P29"/>
+      <c r="Q29" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17">
       <c r="A30">
         <v>282</v>
       </c>
@@ -1857,33 +2476,46 @@
         <v>280</v>
       </c>
       <c r="C30" t="s">
-        <v>96</v>
-      </c>
-      <c r="D30">
+        <v>157</v>
+      </c>
+      <c r="D30" t="s">
+        <v>158</v>
+      </c>
+      <c r="E30">
         <v>29</v>
       </c>
-      <c r="E30" t="s">
-        <v>97</v>
-      </c>
       <c r="F30" t="s">
-        <v>98</v>
+        <v>159</v>
       </c>
       <c r="G30" t="s">
-        <v>96</v>
+        <v>160</v>
       </c>
       <c r="H30" t="s">
-        <v>98</v>
-      </c>
-      <c r="I30"/>
-      <c r="J30">
-        <v>0</v>
-      </c>
-      <c r="K30"/>
+        <v>161</v>
+      </c>
+      <c r="I30" t="s">
+        <v>157</v>
+      </c>
+      <c r="J30" t="s">
+        <v>158</v>
+      </c>
+      <c r="K30" t="s">
+        <v>160</v>
+      </c>
       <c r="L30" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12">
+        <v>161</v>
+      </c>
+      <c r="M30"/>
+      <c r="N30"/>
+      <c r="O30">
+        <v>0</v>
+      </c>
+      <c r="P30"/>
+      <c r="Q30" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17">
       <c r="A31">
         <v>290</v>
       </c>
@@ -1891,33 +2523,46 @@
         <v>0</v>
       </c>
       <c r="C31" t="s">
-        <v>99</v>
-      </c>
-      <c r="D31">
+        <v>162</v>
+      </c>
+      <c r="D31" t="s">
+        <v>163</v>
+      </c>
+      <c r="E31">
         <v>30</v>
       </c>
-      <c r="E31" t="s">
-        <v>100</v>
-      </c>
       <c r="F31" t="s">
-        <v>101</v>
+        <v>164</v>
       </c>
       <c r="G31" t="s">
-        <v>99</v>
+        <v>165</v>
       </c>
       <c r="H31" t="s">
-        <v>101</v>
-      </c>
-      <c r="I31"/>
-      <c r="J31">
-        <v>0</v>
-      </c>
-      <c r="K31"/>
+        <v>166</v>
+      </c>
+      <c r="I31" t="s">
+        <v>162</v>
+      </c>
+      <c r="J31" t="s">
+        <v>163</v>
+      </c>
+      <c r="K31" t="s">
+        <v>165</v>
+      </c>
       <c r="L31" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12">
+        <v>166</v>
+      </c>
+      <c r="M31"/>
+      <c r="N31"/>
+      <c r="O31">
+        <v>0</v>
+      </c>
+      <c r="P31"/>
+      <c r="Q31" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17">
       <c r="A32">
         <v>330</v>
       </c>
@@ -1925,33 +2570,46 @@
         <v>0</v>
       </c>
       <c r="C32" t="s">
-        <v>102</v>
-      </c>
-      <c r="D32">
+        <v>167</v>
+      </c>
+      <c r="D32" t="s">
+        <v>168</v>
+      </c>
+      <c r="E32">
         <v>31</v>
       </c>
-      <c r="E32" t="s">
-        <v>103</v>
-      </c>
       <c r="F32" t="s">
-        <v>104</v>
+        <v>169</v>
       </c>
       <c r="G32" t="s">
-        <v>102</v>
+        <v>170</v>
       </c>
       <c r="H32" t="s">
-        <v>104</v>
-      </c>
-      <c r="I32"/>
-      <c r="J32">
-        <v>0</v>
-      </c>
-      <c r="K32"/>
+        <v>171</v>
+      </c>
+      <c r="I32" t="s">
+        <v>167</v>
+      </c>
+      <c r="J32" t="s">
+        <v>168</v>
+      </c>
+      <c r="K32" t="s">
+        <v>170</v>
+      </c>
       <c r="L32" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12">
+        <v>171</v>
+      </c>
+      <c r="M32"/>
+      <c r="N32"/>
+      <c r="O32">
+        <v>0</v>
+      </c>
+      <c r="P32"/>
+      <c r="Q32" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17">
       <c r="A33">
         <v>331</v>
       </c>
@@ -1959,33 +2617,46 @@
         <v>700</v>
       </c>
       <c r="C33" t="s">
-        <v>105</v>
-      </c>
-      <c r="D33">
+        <v>172</v>
+      </c>
+      <c r="D33" t="s">
+        <v>173</v>
+      </c>
+      <c r="E33">
         <v>32</v>
       </c>
-      <c r="E33" t="s">
-        <v>106</v>
-      </c>
       <c r="F33" t="s">
-        <v>107</v>
+        <v>174</v>
       </c>
       <c r="G33" t="s">
-        <v>105</v>
+        <v>175</v>
       </c>
       <c r="H33" t="s">
-        <v>107</v>
-      </c>
-      <c r="I33"/>
-      <c r="J33">
-        <v>0</v>
-      </c>
-      <c r="K33"/>
+        <v>176</v>
+      </c>
+      <c r="I33" t="s">
+        <v>172</v>
+      </c>
+      <c r="J33" t="s">
+        <v>173</v>
+      </c>
+      <c r="K33" t="s">
+        <v>175</v>
+      </c>
       <c r="L33" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12">
+        <v>176</v>
+      </c>
+      <c r="M33"/>
+      <c r="N33"/>
+      <c r="O33">
+        <v>0</v>
+      </c>
+      <c r="P33"/>
+      <c r="Q33" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17">
       <c r="A34">
         <v>332</v>
       </c>
@@ -1993,33 +2664,46 @@
         <v>700</v>
       </c>
       <c r="C34" t="s">
-        <v>108</v>
-      </c>
-      <c r="D34">
+        <v>177</v>
+      </c>
+      <c r="D34" t="s">
+        <v>178</v>
+      </c>
+      <c r="E34">
         <v>33</v>
       </c>
-      <c r="E34" t="s">
-        <v>109</v>
-      </c>
       <c r="F34" t="s">
-        <v>110</v>
+        <v>179</v>
       </c>
       <c r="G34" t="s">
-        <v>108</v>
+        <v>180</v>
       </c>
       <c r="H34" t="s">
-        <v>110</v>
-      </c>
-      <c r="I34"/>
-      <c r="J34">
-        <v>0</v>
-      </c>
-      <c r="K34"/>
+        <v>181</v>
+      </c>
+      <c r="I34" t="s">
+        <v>177</v>
+      </c>
+      <c r="J34" t="s">
+        <v>178</v>
+      </c>
+      <c r="K34" t="s">
+        <v>180</v>
+      </c>
       <c r="L34" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12">
+        <v>181</v>
+      </c>
+      <c r="M34"/>
+      <c r="N34"/>
+      <c r="O34">
+        <v>0</v>
+      </c>
+      <c r="P34"/>
+      <c r="Q34" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17">
       <c r="A35">
         <v>400</v>
       </c>
@@ -2027,33 +2711,46 @@
         <v>0</v>
       </c>
       <c r="C35" t="s">
-        <v>111</v>
-      </c>
-      <c r="D35">
+        <v>182</v>
+      </c>
+      <c r="D35" t="s">
+        <v>183</v>
+      </c>
+      <c r="E35">
         <v>34</v>
       </c>
-      <c r="E35" t="s">
-        <v>112</v>
-      </c>
       <c r="F35" t="s">
-        <v>111</v>
+        <v>184</v>
       </c>
       <c r="G35" t="s">
-        <v>111</v>
+        <v>182</v>
       </c>
       <c r="H35" t="s">
-        <v>111</v>
-      </c>
-      <c r="I35"/>
-      <c r="J35">
-        <v>0</v>
-      </c>
-      <c r="K35"/>
+        <v>183</v>
+      </c>
+      <c r="I35" t="s">
+        <v>182</v>
+      </c>
+      <c r="J35" t="s">
+        <v>183</v>
+      </c>
+      <c r="K35" t="s">
+        <v>182</v>
+      </c>
       <c r="L35" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12">
+        <v>183</v>
+      </c>
+      <c r="M35"/>
+      <c r="N35"/>
+      <c r="O35">
+        <v>0</v>
+      </c>
+      <c r="P35"/>
+      <c r="Q35" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17">
       <c r="A36">
         <v>401</v>
       </c>
@@ -2061,33 +2758,46 @@
         <v>400</v>
       </c>
       <c r="C36" t="s">
-        <v>113</v>
-      </c>
-      <c r="D36">
+        <v>185</v>
+      </c>
+      <c r="D36" t="s">
+        <v>186</v>
+      </c>
+      <c r="E36">
         <v>35</v>
       </c>
-      <c r="E36" t="s">
-        <v>114</v>
-      </c>
       <c r="F36" t="s">
-        <v>113</v>
+        <v>187</v>
       </c>
       <c r="G36" t="s">
-        <v>113</v>
+        <v>185</v>
       </c>
       <c r="H36" t="s">
-        <v>113</v>
-      </c>
-      <c r="I36"/>
-      <c r="J36">
-        <v>0</v>
-      </c>
-      <c r="K36"/>
+        <v>186</v>
+      </c>
+      <c r="I36" t="s">
+        <v>185</v>
+      </c>
+      <c r="J36" t="s">
+        <v>186</v>
+      </c>
+      <c r="K36" t="s">
+        <v>185</v>
+      </c>
       <c r="L36" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12">
+        <v>186</v>
+      </c>
+      <c r="M36"/>
+      <c r="N36"/>
+      <c r="O36">
+        <v>0</v>
+      </c>
+      <c r="P36"/>
+      <c r="Q36" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17">
       <c r="A37">
         <v>402</v>
       </c>
@@ -2095,33 +2805,46 @@
         <v>400</v>
       </c>
       <c r="C37" t="s">
-        <v>115</v>
-      </c>
-      <c r="D37">
+        <v>188</v>
+      </c>
+      <c r="D37" t="s">
+        <v>189</v>
+      </c>
+      <c r="E37">
         <v>36</v>
       </c>
-      <c r="E37" t="s">
-        <v>116</v>
-      </c>
       <c r="F37" t="s">
-        <v>115</v>
+        <v>190</v>
       </c>
       <c r="G37" t="s">
-        <v>115</v>
+        <v>188</v>
       </c>
       <c r="H37" t="s">
-        <v>115</v>
-      </c>
-      <c r="I37"/>
-      <c r="J37">
-        <v>0</v>
-      </c>
-      <c r="K37"/>
+        <v>189</v>
+      </c>
+      <c r="I37" t="s">
+        <v>188</v>
+      </c>
+      <c r="J37" t="s">
+        <v>189</v>
+      </c>
+      <c r="K37" t="s">
+        <v>188</v>
+      </c>
       <c r="L37" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12">
+        <v>189</v>
+      </c>
+      <c r="M37"/>
+      <c r="N37"/>
+      <c r="O37">
+        <v>0</v>
+      </c>
+      <c r="P37"/>
+      <c r="Q37" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17">
       <c r="A38">
         <v>403</v>
       </c>
@@ -2129,33 +2852,46 @@
         <v>400</v>
       </c>
       <c r="C38" t="s">
-        <v>117</v>
-      </c>
-      <c r="D38">
+        <v>191</v>
+      </c>
+      <c r="D38" t="s">
+        <v>192</v>
+      </c>
+      <c r="E38">
         <v>37</v>
       </c>
-      <c r="E38" t="s">
-        <v>118</v>
-      </c>
       <c r="F38" t="s">
-        <v>117</v>
+        <v>193</v>
       </c>
       <c r="G38" t="s">
-        <v>117</v>
+        <v>191</v>
       </c>
       <c r="H38" t="s">
-        <v>117</v>
-      </c>
-      <c r="I38"/>
-      <c r="J38">
-        <v>0</v>
-      </c>
-      <c r="K38"/>
+        <v>192</v>
+      </c>
+      <c r="I38" t="s">
+        <v>191</v>
+      </c>
+      <c r="J38" t="s">
+        <v>192</v>
+      </c>
+      <c r="K38" t="s">
+        <v>191</v>
+      </c>
       <c r="L38" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12">
+        <v>192</v>
+      </c>
+      <c r="M38"/>
+      <c r="N38"/>
+      <c r="O38">
+        <v>0</v>
+      </c>
+      <c r="P38"/>
+      <c r="Q38" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17">
       <c r="A39">
         <v>405</v>
       </c>
@@ -2163,33 +2899,46 @@
         <v>400</v>
       </c>
       <c r="C39" t="s">
-        <v>119</v>
-      </c>
-      <c r="D39">
+        <v>194</v>
+      </c>
+      <c r="D39" t="s">
+        <v>195</v>
+      </c>
+      <c r="E39">
         <v>38</v>
       </c>
-      <c r="E39" t="s">
-        <v>120</v>
-      </c>
       <c r="F39" t="s">
-        <v>119</v>
+        <v>196</v>
       </c>
       <c r="G39" t="s">
-        <v>119</v>
+        <v>194</v>
       </c>
       <c r="H39" t="s">
-        <v>119</v>
-      </c>
-      <c r="I39"/>
-      <c r="J39">
-        <v>0</v>
-      </c>
-      <c r="K39"/>
+        <v>195</v>
+      </c>
+      <c r="I39" t="s">
+        <v>194</v>
+      </c>
+      <c r="J39" t="s">
+        <v>195</v>
+      </c>
+      <c r="K39" t="s">
+        <v>194</v>
+      </c>
       <c r="L39" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12">
+        <v>195</v>
+      </c>
+      <c r="M39"/>
+      <c r="N39"/>
+      <c r="O39">
+        <v>0</v>
+      </c>
+      <c r="P39"/>
+      <c r="Q39" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17">
       <c r="A40">
         <v>406</v>
       </c>
@@ -2197,33 +2946,46 @@
         <v>400</v>
       </c>
       <c r="C40" t="s">
-        <v>121</v>
-      </c>
-      <c r="D40">
+        <v>197</v>
+      </c>
+      <c r="D40" t="s">
+        <v>198</v>
+      </c>
+      <c r="E40">
         <v>39</v>
       </c>
-      <c r="E40" t="s">
-        <v>122</v>
-      </c>
       <c r="F40" t="s">
-        <v>121</v>
+        <v>199</v>
       </c>
       <c r="G40" t="s">
-        <v>121</v>
+        <v>197</v>
       </c>
       <c r="H40" t="s">
-        <v>121</v>
-      </c>
-      <c r="I40"/>
-      <c r="J40">
-        <v>0</v>
-      </c>
-      <c r="K40"/>
+        <v>198</v>
+      </c>
+      <c r="I40" t="s">
+        <v>197</v>
+      </c>
+      <c r="J40" t="s">
+        <v>198</v>
+      </c>
+      <c r="K40" t="s">
+        <v>197</v>
+      </c>
       <c r="L40" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12">
+        <v>198</v>
+      </c>
+      <c r="M40"/>
+      <c r="N40"/>
+      <c r="O40">
+        <v>0</v>
+      </c>
+      <c r="P40"/>
+      <c r="Q40" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17">
       <c r="A41">
         <v>407</v>
       </c>
@@ -2231,33 +2993,46 @@
         <v>400</v>
       </c>
       <c r="C41" t="s">
-        <v>123</v>
-      </c>
-      <c r="D41">
+        <v>200</v>
+      </c>
+      <c r="D41" t="s">
+        <v>201</v>
+      </c>
+      <c r="E41">
         <v>40</v>
       </c>
-      <c r="E41" t="s">
-        <v>124</v>
-      </c>
       <c r="F41" t="s">
-        <v>123</v>
+        <v>202</v>
       </c>
       <c r="G41" t="s">
-        <v>123</v>
+        <v>200</v>
       </c>
       <c r="H41" t="s">
-        <v>123</v>
-      </c>
-      <c r="I41"/>
-      <c r="J41">
-        <v>0</v>
-      </c>
-      <c r="K41"/>
+        <v>201</v>
+      </c>
+      <c r="I41" t="s">
+        <v>200</v>
+      </c>
+      <c r="J41" t="s">
+        <v>201</v>
+      </c>
+      <c r="K41" t="s">
+        <v>200</v>
+      </c>
       <c r="L41" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12">
+        <v>201</v>
+      </c>
+      <c r="M41"/>
+      <c r="N41"/>
+      <c r="O41">
+        <v>0</v>
+      </c>
+      <c r="P41"/>
+      <c r="Q41" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17">
       <c r="A42">
         <v>500</v>
       </c>
@@ -2265,26 +3040,35 @@
         <v>0</v>
       </c>
       <c r="C42" t="s">
-        <v>125</v>
-      </c>
-      <c r="D42">
+        <v>203</v>
+      </c>
+      <c r="D42" t="s">
+        <v>204</v>
+      </c>
+      <c r="E42">
         <v>41</v>
       </c>
-      <c r="E42" t="s">
-        <v>126</v>
-      </c>
-      <c r="F42"/>
-      <c r="G42" t="s">
-        <v>125</v>
-      </c>
+      <c r="F42" t="s">
+        <v>205</v>
+      </c>
+      <c r="G42"/>
       <c r="H42"/>
-      <c r="I42"/>
-      <c r="J42">
-        <v>0</v>
+      <c r="I42" t="s">
+        <v>203</v>
+      </c>
+      <c r="J42" t="s">
+        <v>204</v>
       </c>
       <c r="K42"/>
-      <c r="L42" t="s">
-        <v>15</v>
+      <c r="L42"/>
+      <c r="M42"/>
+      <c r="N42"/>
+      <c r="O42">
+        <v>0</v>
+      </c>
+      <c r="P42"/>
+      <c r="Q42" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -2309,21 +3093,24 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>127</v>
+        <v>206</v>
       </c>
       <c r="C1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
+        <v>207</v>
+      </c>
+      <c r="D1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2">
         <v>100</v>
       </c>
@@ -2331,10 +3118,13 @@
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+        <v>209</v>
+      </c>
+      <c r="D2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3">
         <v>101</v>
       </c>
@@ -2342,10 +3132,13 @@
         <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
+        <v>210</v>
+      </c>
+      <c r="D3" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4">
         <v>102</v>
       </c>
@@ -2353,10 +3146,13 @@
         <v>0</v>
       </c>
       <c r="C4" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
+        <v>211</v>
+      </c>
+      <c r="D4" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5">
         <v>103</v>
       </c>
@@ -2364,10 +3160,13 @@
         <v>0</v>
       </c>
       <c r="C5" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
+        <v>212</v>
+      </c>
+      <c r="D5" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6">
         <v>110</v>
       </c>
@@ -2375,10 +3174,13 @@
         <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
+        <v>213</v>
+      </c>
+      <c r="D6" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7">
         <v>120</v>
       </c>
@@ -2386,10 +3188,13 @@
         <v>0</v>
       </c>
       <c r="C7" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
+        <v>214</v>
+      </c>
+      <c r="D7" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8">
         <v>121</v>
       </c>
@@ -2397,10 +3202,13 @@
         <v>0</v>
       </c>
       <c r="C8" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
+        <v>215</v>
+      </c>
+      <c r="D8" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
       <c r="A9">
         <v>122</v>
       </c>
@@ -2408,10 +3216,13 @@
         <v>0</v>
       </c>
       <c r="C9" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
+        <v>216</v>
+      </c>
+      <c r="D9" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10">
         <v>123</v>
       </c>
@@ -2419,10 +3230,13 @@
         <v>0</v>
       </c>
       <c r="C10" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
+        <v>217</v>
+      </c>
+      <c r="D10" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
       <c r="A11">
         <v>124</v>
       </c>
@@ -2430,10 +3244,13 @@
         <v>0</v>
       </c>
       <c r="C11" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
+        <v>218</v>
+      </c>
+      <c r="D11" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
       <c r="A12">
         <v>130</v>
       </c>
@@ -2441,10 +3258,13 @@
         <v>0</v>
       </c>
       <c r="C12" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
+        <v>219</v>
+      </c>
+      <c r="D12" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
       <c r="A13">
         <v>140</v>
       </c>
@@ -2452,10 +3272,13 @@
         <v>0</v>
       </c>
       <c r="C13" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
+        <v>220</v>
+      </c>
+      <c r="D13" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
       <c r="A14">
         <v>141</v>
       </c>
@@ -2463,10 +3286,13 @@
         <v>0</v>
       </c>
       <c r="C14" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
+        <v>221</v>
+      </c>
+      <c r="D14" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
       <c r="A15">
         <v>142</v>
       </c>
@@ -2474,10 +3300,13 @@
         <v>0</v>
       </c>
       <c r="C15" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
+        <v>222</v>
+      </c>
+      <c r="D15" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
       <c r="A16">
         <v>150</v>
       </c>
@@ -2485,10 +3314,13 @@
         <v>0</v>
       </c>
       <c r="C16" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3">
+        <v>223</v>
+      </c>
+      <c r="D16" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
       <c r="A17">
         <v>160</v>
       </c>
@@ -2496,10 +3328,13 @@
         <v>0</v>
       </c>
       <c r="C17" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3">
+        <v>224</v>
+      </c>
+      <c r="D17" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
       <c r="A18">
         <v>170</v>
       </c>
@@ -2507,10 +3342,13 @@
         <v>0</v>
       </c>
       <c r="C18" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
+        <v>225</v>
+      </c>
+      <c r="D18" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
       <c r="A19">
         <v>180</v>
       </c>
@@ -2518,10 +3356,13 @@
         <v>0</v>
       </c>
       <c r="C19" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3">
+        <v>226</v>
+      </c>
+      <c r="D19" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
       <c r="A20">
         <v>190</v>
       </c>
@@ -2529,10 +3370,13 @@
         <v>0</v>
       </c>
       <c r="C20" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3">
+        <v>227</v>
+      </c>
+      <c r="D20" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
       <c r="A21">
         <v>200</v>
       </c>
@@ -2540,10 +3384,13 @@
         <v>0</v>
       </c>
       <c r="C21" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
+        <v>228</v>
+      </c>
+      <c r="D21" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
       <c r="A22">
         <v>210</v>
       </c>
@@ -2551,10 +3398,13 @@
         <v>0</v>
       </c>
       <c r="C22" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3">
+        <v>229</v>
+      </c>
+      <c r="D22" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
       <c r="A23">
         <v>220</v>
       </c>
@@ -2562,10 +3412,13 @@
         <v>0</v>
       </c>
       <c r="C23" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3">
+        <v>230</v>
+      </c>
+      <c r="D23" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
       <c r="A24">
         <v>230</v>
       </c>
@@ -2573,10 +3426,13 @@
         <v>0</v>
       </c>
       <c r="C24" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3">
+        <v>231</v>
+      </c>
+      <c r="D24" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
       <c r="A25">
         <v>240</v>
       </c>
@@ -2584,10 +3440,13 @@
         <v>0</v>
       </c>
       <c r="C25" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3">
+        <v>232</v>
+      </c>
+      <c r="D25" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
       <c r="A26">
         <v>250</v>
       </c>
@@ -2595,10 +3454,13 @@
         <v>0</v>
       </c>
       <c r="C26" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3">
+        <v>233</v>
+      </c>
+      <c r="D26" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
       <c r="A27">
         <v>270</v>
       </c>
@@ -2606,10 +3468,13 @@
         <v>0</v>
       </c>
       <c r="C27" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3">
+        <v>234</v>
+      </c>
+      <c r="D27" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
       <c r="A28">
         <v>280</v>
       </c>
@@ -2617,10 +3482,13 @@
         <v>0</v>
       </c>
       <c r="C28" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3">
+        <v>235</v>
+      </c>
+      <c r="D28" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
       <c r="A29">
         <v>281</v>
       </c>
@@ -2628,10 +3496,13 @@
         <v>0</v>
       </c>
       <c r="C29" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3">
+        <v>236</v>
+      </c>
+      <c r="D29" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
       <c r="A30">
         <v>282</v>
       </c>
@@ -2639,10 +3510,13 @@
         <v>0</v>
       </c>
       <c r="C30" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3">
+        <v>237</v>
+      </c>
+      <c r="D30" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
       <c r="A31">
         <v>290</v>
       </c>
@@ -2650,10 +3524,13 @@
         <v>0</v>
       </c>
       <c r="C31" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3">
+        <v>238</v>
+      </c>
+      <c r="D31" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
       <c r="A32">
         <v>330</v>
       </c>
@@ -2661,10 +3538,13 @@
         <v>0</v>
       </c>
       <c r="C32" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3">
+        <v>239</v>
+      </c>
+      <c r="D32" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
       <c r="A33">
         <v>331</v>
       </c>
@@ -2672,10 +3552,13 @@
         <v>0</v>
       </c>
       <c r="C33" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3">
+        <v>240</v>
+      </c>
+      <c r="D33" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
       <c r="A34">
         <v>332</v>
       </c>
@@ -2683,10 +3566,13 @@
         <v>0</v>
       </c>
       <c r="C34" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3">
+        <v>241</v>
+      </c>
+      <c r="D34" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
       <c r="A35">
         <v>400</v>
       </c>
@@ -2694,10 +3580,13 @@
         <v>0</v>
       </c>
       <c r="C35" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
+        <v>242</v>
+      </c>
+      <c r="D35" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
       <c r="A36">
         <v>401</v>
       </c>
@@ -2705,10 +3594,13 @@
         <v>0</v>
       </c>
       <c r="C36" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3">
+        <v>243</v>
+      </c>
+      <c r="D36" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
       <c r="A37">
         <v>402</v>
       </c>
@@ -2716,10 +3608,13 @@
         <v>0</v>
       </c>
       <c r="C37" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3">
+        <v>244</v>
+      </c>
+      <c r="D37" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
       <c r="A38">
         <v>403</v>
       </c>
@@ -2727,10 +3622,13 @@
         <v>0</v>
       </c>
       <c r="C38" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3">
+        <v>245</v>
+      </c>
+      <c r="D38" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
       <c r="A39">
         <v>405</v>
       </c>
@@ -2738,10 +3636,13 @@
         <v>0</v>
       </c>
       <c r="C39" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3">
+        <v>246</v>
+      </c>
+      <c r="D39" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
       <c r="A40">
         <v>406</v>
       </c>
@@ -2749,10 +3650,13 @@
         <v>0</v>
       </c>
       <c r="C40" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3">
+        <v>247</v>
+      </c>
+      <c r="D40" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
       <c r="A41">
         <v>407</v>
       </c>
@@ -2760,8 +3664,21 @@
         <v>0</v>
       </c>
       <c r="C41" t="s">
-        <v>168</v>
-      </c>
+        <v>248</v>
+      </c>
+      <c r="D41" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42">
+        <v>500</v>
+      </c>
+      <c r="B42">
+        <v>0</v>
+      </c>
+      <c r="C42"/>
+      <c r="D42"/>
     </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>

</xml_diff>

<commit_message>
fix: point flower subcategories to 330 and rebuild categories xls
</commit_message>
<xml_diff>
--- a/shared/data/categories_import.xlsx
+++ b/shared/data/categories_import.xlsx
@@ -2738,7 +2738,7 @@
         <v>331</v>
       </c>
       <c r="B33">
-        <v>300</v>
+        <v>330</v>
       </c>
       <c r="C33" t="s">
         <v>172</v>
@@ -2789,7 +2789,7 @@
         <v>332</v>
       </c>
       <c r="B34">
-        <v>300</v>
+        <v>330</v>
       </c>
       <c r="C34" t="s">
         <v>177</v>

</xml_diff>